<commit_message>
state: bot run 2026-09-08T04:53 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3238,6 +3238,694 @@
         <v>0</v>
       </c>
       <c r="K65" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 168.74 &lt;= Upper 170.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>230.36</v>
+      </c>
+      <c r="E66" t="n">
+        <v>232.35</v>
+      </c>
+      <c r="F66" t="n">
+        <v>232.35</v>
+      </c>
+      <c r="G66" t="n">
+        <v>222.89</v>
+      </c>
+      <c r="H66" t="n">
+        <v>219.04</v>
+      </c>
+      <c r="I66" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J66" t="b">
+        <v>0</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 230.36 &lt;= Upper 232.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>354.08</v>
+      </c>
+      <c r="E67" t="n">
+        <v>373.23</v>
+      </c>
+      <c r="F67" t="n">
+        <v>373.23</v>
+      </c>
+      <c r="G67" t="n">
+        <v>357.35</v>
+      </c>
+      <c r="H67" t="n">
+        <v>351.67</v>
+      </c>
+      <c r="I67" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="J67" t="b">
+        <v>0</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 354.08 &lt;= Upper 373.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>319.97</v>
+      </c>
+      <c r="E68" t="n">
+        <v>328.06</v>
+      </c>
+      <c r="F68" t="n">
+        <v>328.06</v>
+      </c>
+      <c r="G68" t="n">
+        <v>319.98</v>
+      </c>
+      <c r="H68" t="n">
+        <v>316.73</v>
+      </c>
+      <c r="I68" t="n">
+        <v>1</v>
+      </c>
+      <c r="J68" t="b">
+        <v>0</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 319.97 &lt;= Upper 328.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>499.7</v>
+      </c>
+      <c r="E69" t="n">
+        <v>516.08</v>
+      </c>
+      <c r="F69" t="n">
+        <v>516.08</v>
+      </c>
+      <c r="G69" t="n">
+        <v>500.48</v>
+      </c>
+      <c r="H69" t="n">
+        <v>488.68</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J69" t="b">
+        <v>0</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 499.70 &lt;= Upper 516.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>616.77</v>
+      </c>
+      <c r="E70" t="n">
+        <v>619.29</v>
+      </c>
+      <c r="F70" t="n">
+        <v>619.29</v>
+      </c>
+      <c r="G70" t="n">
+        <v>589.64</v>
+      </c>
+      <c r="H70" t="n">
+        <v>583.6</v>
+      </c>
+      <c r="I70" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" t="b">
+        <v>0</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 616.77 &lt;= Upper 619.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>258.51</v>
+      </c>
+      <c r="E71" t="n">
+        <v>273.63</v>
+      </c>
+      <c r="F71" t="n">
+        <v>273.63</v>
+      </c>
+      <c r="G71" t="n">
+        <v>258.96</v>
+      </c>
+      <c r="H71" t="n">
+        <v>259.54</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J71" t="b">
+        <v>0</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 258.96 &lt;= EMA21 259.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>338.46</v>
+      </c>
+      <c r="E72" t="n">
+        <v>352.9</v>
+      </c>
+      <c r="F72" t="n">
+        <v>352.9</v>
+      </c>
+      <c r="G72" t="n">
+        <v>340.57</v>
+      </c>
+      <c r="H72" t="n">
+        <v>343.38</v>
+      </c>
+      <c r="I72" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J72" t="b">
+        <v>0</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 340.57 &lt;= EMA21 343.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>477.57</v>
+      </c>
+      <c r="E73" t="n">
+        <v>505.22</v>
+      </c>
+      <c r="F73" t="n">
+        <v>505.22</v>
+      </c>
+      <c r="G73" t="n">
+        <v>468.28</v>
+      </c>
+      <c r="H73" t="n">
+        <v>475.5</v>
+      </c>
+      <c r="I73" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J73" t="b">
+        <v>0</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 468.28 &lt;= EMA21 475.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="E74" t="n">
+        <v>84.38</v>
+      </c>
+      <c r="F74" t="n">
+        <v>84.38</v>
+      </c>
+      <c r="G74" t="n">
+        <v>80.62</v>
+      </c>
+      <c r="H74" t="n">
+        <v>79.13</v>
+      </c>
+      <c r="I74" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J74" t="b">
+        <v>0</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 78.25 &lt;= Upper 84.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>174.33</v>
+      </c>
+      <c r="E75" t="n">
+        <v>187.21</v>
+      </c>
+      <c r="F75" t="n">
+        <v>187.21</v>
+      </c>
+      <c r="G75" t="n">
+        <v>177.88</v>
+      </c>
+      <c r="H75" t="n">
+        <v>171.96</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J75" t="b">
+        <v>0</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.33 &lt;= Upper 187.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>357.9</v>
+      </c>
+      <c r="E76" t="n">
+        <v>424.09</v>
+      </c>
+      <c r="F76" t="n">
+        <v>424.09</v>
+      </c>
+      <c r="G76" t="n">
+        <v>365.27</v>
+      </c>
+      <c r="H76" t="n">
+        <v>374.12</v>
+      </c>
+      <c r="I76" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.27 &lt;= EMA21 374.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>184.64</v>
+      </c>
+      <c r="E77" t="n">
+        <v>204.15</v>
+      </c>
+      <c r="F77" t="n">
+        <v>204.15</v>
+      </c>
+      <c r="G77" t="n">
+        <v>181.51</v>
+      </c>
+      <c r="H77" t="n">
+        <v>173.86</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J77" t="b">
+        <v>0</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 184.64 &lt;= Upper 204.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>252.09</v>
+      </c>
+      <c r="E78" t="n">
+        <v>282.59</v>
+      </c>
+      <c r="F78" t="n">
+        <v>282.59</v>
+      </c>
+      <c r="G78" t="n">
+        <v>244.99</v>
+      </c>
+      <c r="H78" t="n">
+        <v>252.3</v>
+      </c>
+      <c r="I78" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J78" t="b">
+        <v>0</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 244.99 &lt;= EMA21 252.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>75.76000000000001</v>
+      </c>
+      <c r="E79" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="F79" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="G79" t="n">
+        <v>76.54000000000001</v>
+      </c>
+      <c r="H79" t="n">
+        <v>76.11</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J79" t="b">
+        <v>0</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 75.76 &lt;= Upper 80.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>39.59</v>
+      </c>
+      <c r="E80" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="F80" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G80" t="n">
+        <v>37.67</v>
+      </c>
+      <c r="H80" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J80" t="b">
+        <v>0</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 39.59 &lt;= Upper 41.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>168.74</v>
+      </c>
+      <c r="E81" t="n">
+        <v>170.32</v>
+      </c>
+      <c r="F81" t="n">
+        <v>170.32</v>
+      </c>
+      <c r="G81" t="n">
+        <v>166.2</v>
+      </c>
+      <c r="H81" t="n">
+        <v>164.92</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J81" t="b">
+        <v>0</v>
+      </c>
+      <c r="K81" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 168.74 &lt;= Upper 170.32)</t>
         </is>
@@ -3907,7 +4595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4089,6 +4777,39 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04:53:12</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-171.28</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-09T04:53 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K481"/>
+  <dimension ref="A1:K581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20912,6 +20912,4252 @@
       <c r="K481" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 104.47 &lt;= Upper 109.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D482" t="n">
+        <v>316.22</v>
+      </c>
+      <c r="E482" t="n">
+        <v>328.33</v>
+      </c>
+      <c r="F482" t="n">
+        <v>328.33</v>
+      </c>
+      <c r="G482" t="n">
+        <v>319.23</v>
+      </c>
+      <c r="H482" t="n">
+        <v>316.68</v>
+      </c>
+      <c r="I482" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J482" t="b">
+        <v>0</v>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 316.22 &lt;= Upper 328.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>493.95</v>
+      </c>
+      <c r="E483" t="n">
+        <v>515.01</v>
+      </c>
+      <c r="F483" t="n">
+        <v>515.01</v>
+      </c>
+      <c r="G483" t="n">
+        <v>499.18</v>
+      </c>
+      <c r="H483" t="n">
+        <v>489.16</v>
+      </c>
+      <c r="I483" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J483" t="b">
+        <v>0</v>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 493.95 &lt;= Upper 515.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>225.73</v>
+      </c>
+      <c r="E484" t="n">
+        <v>232.95</v>
+      </c>
+      <c r="F484" t="n">
+        <v>232.95</v>
+      </c>
+      <c r="G484" t="n">
+        <v>223.46</v>
+      </c>
+      <c r="H484" t="n">
+        <v>219.65</v>
+      </c>
+      <c r="I484" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J484" t="b">
+        <v>0</v>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 225.73 &lt;= Upper 232.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>338.36</v>
+      </c>
+      <c r="E485" t="n">
+        <v>349.61</v>
+      </c>
+      <c r="F485" t="n">
+        <v>349.61</v>
+      </c>
+      <c r="G485" t="n">
+        <v>340.13</v>
+      </c>
+      <c r="H485" t="n">
+        <v>342.93</v>
+      </c>
+      <c r="I485" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J485" t="b">
+        <v>0</v>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 340.13 &lt;= EMA21 342.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>335.38</v>
+      </c>
+      <c r="E486" t="n">
+        <v>347.06</v>
+      </c>
+      <c r="F486" t="n">
+        <v>347.06</v>
+      </c>
+      <c r="G486" t="n">
+        <v>336.96</v>
+      </c>
+      <c r="H486" t="n">
+        <v>340.12</v>
+      </c>
+      <c r="I486" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J486" t="b">
+        <v>0</v>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 336.96 &lt;= EMA21 340.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>256.97</v>
+      </c>
+      <c r="E487" t="n">
+        <v>270.01</v>
+      </c>
+      <c r="F487" t="n">
+        <v>270.01</v>
+      </c>
+      <c r="G487" t="n">
+        <v>258.56</v>
+      </c>
+      <c r="H487" t="n">
+        <v>259.3</v>
+      </c>
+      <c r="I487" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J487" t="b">
+        <v>0</v>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 258.56 &lt;= EMA21 259.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>613.48</v>
+      </c>
+      <c r="E488" t="n">
+        <v>622.62</v>
+      </c>
+      <c r="F488" t="n">
+        <v>622.62</v>
+      </c>
+      <c r="G488" t="n">
+        <v>594.41</v>
+      </c>
+      <c r="H488" t="n">
+        <v>586.3200000000001</v>
+      </c>
+      <c r="I488" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J488" t="b">
+        <v>0</v>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 613.48 &lt;= Upper 622.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D489" t="n">
+        <v>368.16</v>
+      </c>
+      <c r="E489" t="n">
+        <v>375.14</v>
+      </c>
+      <c r="F489" t="n">
+        <v>375.14</v>
+      </c>
+      <c r="G489" t="n">
+        <v>359.51</v>
+      </c>
+      <c r="H489" t="n">
+        <v>353.17</v>
+      </c>
+      <c r="I489" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J489" t="b">
+        <v>0</v>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 368.16 &lt;= Upper 375.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D490" t="n">
+        <v>368.56</v>
+      </c>
+      <c r="E490" t="n">
+        <v>416.56</v>
+      </c>
+      <c r="F490" t="n">
+        <v>416.56</v>
+      </c>
+      <c r="G490" t="n">
+        <v>365.93</v>
+      </c>
+      <c r="H490" t="n">
+        <v>373.62</v>
+      </c>
+      <c r="I490" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J490" t="b">
+        <v>0</v>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.93 &lt;= EMA21 373.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D491" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="E491" t="n">
+        <v>160.64</v>
+      </c>
+      <c r="F491" t="n">
+        <v>160.64</v>
+      </c>
+      <c r="G491" t="n">
+        <v>152.61</v>
+      </c>
+      <c r="H491" t="n">
+        <v>148.52</v>
+      </c>
+      <c r="I491" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J491" t="b">
+        <v>1</v>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>249.12</v>
+      </c>
+      <c r="E492" t="n">
+        <v>280.18</v>
+      </c>
+      <c r="F492" t="n">
+        <v>280.18</v>
+      </c>
+      <c r="G492" t="n">
+        <v>247.58</v>
+      </c>
+      <c r="H492" t="n">
+        <v>228.26</v>
+      </c>
+      <c r="I492" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J492" t="b">
+        <v>0</v>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 249.12 &lt;= Upper 280.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>257.26</v>
+      </c>
+      <c r="E493" t="n">
+        <v>296.34</v>
+      </c>
+      <c r="F493" t="n">
+        <v>296.34</v>
+      </c>
+      <c r="G493" t="n">
+        <v>274.76</v>
+      </c>
+      <c r="H493" t="n">
+        <v>270.99</v>
+      </c>
+      <c r="I493" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J493" t="b">
+        <v>0</v>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 257.26 &lt;= Upper 296.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>505.74</v>
+      </c>
+      <c r="E494" t="n">
+        <v>509.82</v>
+      </c>
+      <c r="F494" t="n">
+        <v>509.82</v>
+      </c>
+      <c r="G494" t="n">
+        <v>475.77</v>
+      </c>
+      <c r="H494" t="n">
+        <v>478.25</v>
+      </c>
+      <c r="I494" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J494" t="b">
+        <v>0</v>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 475.77 &lt;= EMA21 478.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>104.47</v>
+      </c>
+      <c r="E495" t="n">
+        <v>106.32</v>
+      </c>
+      <c r="F495" t="n">
+        <v>106.32</v>
+      </c>
+      <c r="G495" t="n">
+        <v>94.3</v>
+      </c>
+      <c r="H495" t="n">
+        <v>94.45999999999999</v>
+      </c>
+      <c r="I495" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J495" t="b">
+        <v>0</v>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 94.30 &lt;= EMA21 94.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>1000.26</v>
+      </c>
+      <c r="E496" t="n">
+        <v>1020.54</v>
+      </c>
+      <c r="F496" t="n">
+        <v>1020.54</v>
+      </c>
+      <c r="G496" t="n">
+        <v>968.05</v>
+      </c>
+      <c r="H496" t="n">
+        <v>948.71</v>
+      </c>
+      <c r="I496" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J496" t="b">
+        <v>0</v>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1000.26 &lt;= Upper 1020.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="E497" t="n">
+        <v>172.39</v>
+      </c>
+      <c r="F497" t="n">
+        <v>172.39</v>
+      </c>
+      <c r="G497" t="n">
+        <v>167.78</v>
+      </c>
+      <c r="H497" t="n">
+        <v>165.76</v>
+      </c>
+      <c r="I497" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="J497" t="b">
+        <v>1</v>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>258.92</v>
+      </c>
+      <c r="E498" t="n">
+        <v>284.02</v>
+      </c>
+      <c r="F498" t="n">
+        <v>284.02</v>
+      </c>
+      <c r="G498" t="n">
+        <v>258.99</v>
+      </c>
+      <c r="H498" t="n">
+        <v>264.84</v>
+      </c>
+      <c r="I498" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J498" t="b">
+        <v>0</v>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 258.99 &lt;= EMA21 264.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>472.79</v>
+      </c>
+      <c r="E499" t="n">
+        <v>552.86</v>
+      </c>
+      <c r="F499" t="n">
+        <v>552.86</v>
+      </c>
+      <c r="G499" t="n">
+        <v>461.87</v>
+      </c>
+      <c r="H499" t="n">
+        <v>481.42</v>
+      </c>
+      <c r="I499" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J499" t="b">
+        <v>0</v>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 461.87 &lt;= EMA21 481.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>320.42</v>
+      </c>
+      <c r="E500" t="n">
+        <v>343.41</v>
+      </c>
+      <c r="F500" t="n">
+        <v>343.41</v>
+      </c>
+      <c r="G500" t="n">
+        <v>305.94</v>
+      </c>
+      <c r="H500" t="n">
+        <v>309.22</v>
+      </c>
+      <c r="I500" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J500" t="b">
+        <v>0</v>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 305.94 &lt;= EMA21 309.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>188.98</v>
+      </c>
+      <c r="E501" t="n">
+        <v>211.92</v>
+      </c>
+      <c r="F501" t="n">
+        <v>211.92</v>
+      </c>
+      <c r="G501" t="n">
+        <v>181.25</v>
+      </c>
+      <c r="H501" t="n">
+        <v>186.11</v>
+      </c>
+      <c r="I501" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J501" t="b">
+        <v>0</v>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 181.25 &lt;= EMA21 186.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>1764.85</v>
+      </c>
+      <c r="E502" t="n">
+        <v>1879.89</v>
+      </c>
+      <c r="F502" t="n">
+        <v>1879.89</v>
+      </c>
+      <c r="G502" t="n">
+        <v>1715.1</v>
+      </c>
+      <c r="H502" t="n">
+        <v>1728.01</v>
+      </c>
+      <c r="I502" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J502" t="b">
+        <v>0</v>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1715.10 &lt;= EMA21 1728.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>363.2</v>
+      </c>
+      <c r="E503" t="n">
+        <v>391.82</v>
+      </c>
+      <c r="F503" t="n">
+        <v>391.82</v>
+      </c>
+      <c r="G503" t="n">
+        <v>362.64</v>
+      </c>
+      <c r="H503" t="n">
+        <v>367.92</v>
+      </c>
+      <c r="I503" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J503" t="b">
+        <v>0</v>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 362.64 &lt;= EMA21 367.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>225.41</v>
+      </c>
+      <c r="E504" t="n">
+        <v>252.08</v>
+      </c>
+      <c r="F504" t="n">
+        <v>252.08</v>
+      </c>
+      <c r="G504" t="n">
+        <v>220.61</v>
+      </c>
+      <c r="H504" t="n">
+        <v>221.31</v>
+      </c>
+      <c r="I504" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J504" t="b">
+        <v>0</v>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 220.61 &lt;= EMA21 221.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>223.87</v>
+      </c>
+      <c r="E505" t="n">
+        <v>235.96</v>
+      </c>
+      <c r="F505" t="n">
+        <v>235.96</v>
+      </c>
+      <c r="G505" t="n">
+        <v>225.58</v>
+      </c>
+      <c r="H505" t="n">
+        <v>229.94</v>
+      </c>
+      <c r="I505" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="J505" t="b">
+        <v>0</v>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.58 &lt;= EMA21 229.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="E506" t="n">
+        <v>84.43000000000001</v>
+      </c>
+      <c r="F506" t="n">
+        <v>84.43000000000001</v>
+      </c>
+      <c r="G506" t="n">
+        <v>73.38</v>
+      </c>
+      <c r="H506" t="n">
+        <v>76.09</v>
+      </c>
+      <c r="I506" t="n">
+        <v>2</v>
+      </c>
+      <c r="J506" t="b">
+        <v>0</v>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 73.38 &lt;= EMA21 76.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>1218.5</v>
+      </c>
+      <c r="E507" t="n">
+        <v>1442.55</v>
+      </c>
+      <c r="F507" t="n">
+        <v>1442.55</v>
+      </c>
+      <c r="G507" t="n">
+        <v>1245.96</v>
+      </c>
+      <c r="H507" t="n">
+        <v>1285.61</v>
+      </c>
+      <c r="I507" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J507" t="b">
+        <v>0</v>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1245.96 &lt;= EMA21 1285.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>75.38</v>
+      </c>
+      <c r="E508" t="n">
+        <v>74</v>
+      </c>
+      <c r="F508" t="n">
+        <v>74</v>
+      </c>
+      <c r="G508" t="n">
+        <v>70.86</v>
+      </c>
+      <c r="H508" t="n">
+        <v>68.81999999999999</v>
+      </c>
+      <c r="I508" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J508" t="b">
+        <v>0</v>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.23x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="E509" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="F509" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="G509" t="n">
+        <v>99.65000000000001</v>
+      </c>
+      <c r="H509" t="n">
+        <v>97.33</v>
+      </c>
+      <c r="I509" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J509" t="b">
+        <v>1</v>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>372.06</v>
+      </c>
+      <c r="E510" t="n">
+        <v>432.17</v>
+      </c>
+      <c r="F510" t="n">
+        <v>432.17</v>
+      </c>
+      <c r="G510" t="n">
+        <v>357.86</v>
+      </c>
+      <c r="H510" t="n">
+        <v>365.47</v>
+      </c>
+      <c r="I510" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J510" t="b">
+        <v>0</v>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 357.86 &lt;= EMA21 365.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>141.09</v>
+      </c>
+      <c r="E511" t="n">
+        <v>166.2</v>
+      </c>
+      <c r="F511" t="n">
+        <v>166.2</v>
+      </c>
+      <c r="G511" t="n">
+        <v>137.49</v>
+      </c>
+      <c r="H511" t="n">
+        <v>139.84</v>
+      </c>
+      <c r="I511" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J511" t="b">
+        <v>0</v>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 137.49 &lt;= EMA21 139.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>73.38</v>
+      </c>
+      <c r="E512" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="F512" t="n">
+        <v>80.68000000000001</v>
+      </c>
+      <c r="G512" t="n">
+        <v>73.69</v>
+      </c>
+      <c r="H512" t="n">
+        <v>75.22</v>
+      </c>
+      <c r="I512" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J512" t="b">
+        <v>0</v>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 73.69 &lt;= EMA21 75.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>40.26</v>
+      </c>
+      <c r="E513" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="F513" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="G513" t="n">
+        <v>38.19</v>
+      </c>
+      <c r="H513" t="n">
+        <v>36.56</v>
+      </c>
+      <c r="I513" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J513" t="b">
+        <v>0</v>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 40.26 &lt;= Upper 41.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>533.88</v>
+      </c>
+      <c r="E514" t="n">
+        <v>533.27</v>
+      </c>
+      <c r="F514" t="n">
+        <v>533.27</v>
+      </c>
+      <c r="G514" t="n">
+        <v>491.52</v>
+      </c>
+      <c r="H514" t="n">
+        <v>470.66</v>
+      </c>
+      <c r="I514" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J514" t="b">
+        <v>0</v>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.78x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>31.17</v>
+      </c>
+      <c r="E515" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="F515" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="G515" t="n">
+        <v>31.17</v>
+      </c>
+      <c r="H515" t="n">
+        <v>30.16</v>
+      </c>
+      <c r="I515" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J515" t="b">
+        <v>0</v>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 31.17 &lt;= Upper 32.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>477.3</v>
+      </c>
+      <c r="E516" t="n">
+        <v>516.08</v>
+      </c>
+      <c r="F516" t="n">
+        <v>516.08</v>
+      </c>
+      <c r="G516" t="n">
+        <v>460.9</v>
+      </c>
+      <c r="H516" t="n">
+        <v>469.37</v>
+      </c>
+      <c r="I516" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J516" t="b">
+        <v>0</v>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 460.90 &lt;= EMA21 469.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D517" t="n">
+        <v>904.38</v>
+      </c>
+      <c r="E517" t="n">
+        <v>968.91</v>
+      </c>
+      <c r="F517" t="n">
+        <v>968.91</v>
+      </c>
+      <c r="G517" t="n">
+        <v>844.61</v>
+      </c>
+      <c r="H517" t="n">
+        <v>846.92</v>
+      </c>
+      <c r="I517" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J517" t="b">
+        <v>0</v>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 844.61 &lt;= EMA21 846.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D518" t="n">
+        <v>194.96</v>
+      </c>
+      <c r="E518" t="n">
+        <v>208.48</v>
+      </c>
+      <c r="F518" t="n">
+        <v>208.48</v>
+      </c>
+      <c r="G518" t="n">
+        <v>192.96</v>
+      </c>
+      <c r="H518" t="n">
+        <v>191.56</v>
+      </c>
+      <c r="I518" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J518" t="b">
+        <v>0</v>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 194.96 &lt;= Upper 208.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>109.17</v>
+      </c>
+      <c r="E519" t="n">
+        <v>119.47</v>
+      </c>
+      <c r="F519" t="n">
+        <v>119.47</v>
+      </c>
+      <c r="G519" t="n">
+        <v>109.95</v>
+      </c>
+      <c r="H519" t="n">
+        <v>111.67</v>
+      </c>
+      <c r="I519" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J519" t="b">
+        <v>0</v>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.95 &lt;= EMA21 111.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>179.03</v>
+      </c>
+      <c r="E520" t="n">
+        <v>195.12</v>
+      </c>
+      <c r="F520" t="n">
+        <v>195.12</v>
+      </c>
+      <c r="G520" t="n">
+        <v>185.7</v>
+      </c>
+      <c r="H520" t="n">
+        <v>181.26</v>
+      </c>
+      <c r="I520" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J520" t="b">
+        <v>0</v>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 179.03 &lt;= Upper 195.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>232.09</v>
+      </c>
+      <c r="E521" t="n">
+        <v>239.58</v>
+      </c>
+      <c r="F521" t="n">
+        <v>239.58</v>
+      </c>
+      <c r="G521" t="n">
+        <v>233.49</v>
+      </c>
+      <c r="H521" t="n">
+        <v>233.67</v>
+      </c>
+      <c r="I521" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J521" t="b">
+        <v>0</v>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 233.49 &lt;= EMA21 233.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>134.21</v>
+      </c>
+      <c r="E522" t="n">
+        <v>149.79</v>
+      </c>
+      <c r="F522" t="n">
+        <v>149.79</v>
+      </c>
+      <c r="G522" t="n">
+        <v>137.97</v>
+      </c>
+      <c r="H522" t="n">
+        <v>131.94</v>
+      </c>
+      <c r="I522" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J522" t="b">
+        <v>0</v>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 134.21 &lt;= Upper 149.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D523" t="n">
+        <v>318.93</v>
+      </c>
+      <c r="E523" t="n">
+        <v>374.96</v>
+      </c>
+      <c r="F523" t="n">
+        <v>374.96</v>
+      </c>
+      <c r="G523" t="n">
+        <v>340.67</v>
+      </c>
+      <c r="H523" t="n">
+        <v>340.68</v>
+      </c>
+      <c r="I523" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J523" t="b">
+        <v>0</v>
+      </c>
+      <c r="K523" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 340.67 &lt;= EMA21 340.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D524" t="n">
+        <v>336.98</v>
+      </c>
+      <c r="E524" t="n">
+        <v>404.41</v>
+      </c>
+      <c r="F524" t="n">
+        <v>404.41</v>
+      </c>
+      <c r="G524" t="n">
+        <v>346.54</v>
+      </c>
+      <c r="H524" t="n">
+        <v>352.3</v>
+      </c>
+      <c r="I524" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J524" t="b">
+        <v>0</v>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 346.54 &lt;= EMA21 352.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D525" t="n">
+        <v>210.02</v>
+      </c>
+      <c r="E525" t="n">
+        <v>237.81</v>
+      </c>
+      <c r="F525" t="n">
+        <v>237.81</v>
+      </c>
+      <c r="G525" t="n">
+        <v>211.2</v>
+      </c>
+      <c r="H525" t="n">
+        <v>208.29</v>
+      </c>
+      <c r="I525" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J525" t="b">
+        <v>0</v>
+      </c>
+      <c r="K525" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 210.02 &lt;= Upper 237.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D526" t="n">
+        <v>335.5</v>
+      </c>
+      <c r="E526" t="n">
+        <v>349.12</v>
+      </c>
+      <c r="F526" t="n">
+        <v>349.12</v>
+      </c>
+      <c r="G526" t="n">
+        <v>330.96</v>
+      </c>
+      <c r="H526" t="n">
+        <v>323.62</v>
+      </c>
+      <c r="I526" t="n">
+        <v>1</v>
+      </c>
+      <c r="J526" t="b">
+        <v>0</v>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 335.50 &lt;= Upper 349.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D527" t="n">
+        <v>170.3</v>
+      </c>
+      <c r="E527" t="n">
+        <v>187.36</v>
+      </c>
+      <c r="F527" t="n">
+        <v>187.36</v>
+      </c>
+      <c r="G527" t="n">
+        <v>176.36</v>
+      </c>
+      <c r="H527" t="n">
+        <v>171.81</v>
+      </c>
+      <c r="I527" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J527" t="b">
+        <v>0</v>
+      </c>
+      <c r="K527" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 170.30 &lt;= Upper 187.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>210.23</v>
+      </c>
+      <c r="E528" t="n">
+        <v>260.73</v>
+      </c>
+      <c r="F528" t="n">
+        <v>260.73</v>
+      </c>
+      <c r="G528" t="n">
+        <v>220.83</v>
+      </c>
+      <c r="H528" t="n">
+        <v>231.14</v>
+      </c>
+      <c r="I528" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J528" t="b">
+        <v>0</v>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 220.83 &lt;= EMA21 231.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>161.94</v>
+      </c>
+      <c r="E529" t="n">
+        <v>193.48</v>
+      </c>
+      <c r="F529" t="n">
+        <v>193.48</v>
+      </c>
+      <c r="G529" t="n">
+        <v>173.88</v>
+      </c>
+      <c r="H529" t="n">
+        <v>173.42</v>
+      </c>
+      <c r="I529" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J529" t="b">
+        <v>0</v>
+      </c>
+      <c r="K529" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 161.94 &lt;= Upper 193.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>284.3</v>
+      </c>
+      <c r="E530" t="n">
+        <v>326</v>
+      </c>
+      <c r="F530" t="n">
+        <v>326</v>
+      </c>
+      <c r="G530" t="n">
+        <v>286.42</v>
+      </c>
+      <c r="H530" t="n">
+        <v>288.57</v>
+      </c>
+      <c r="I530" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J530" t="b">
+        <v>0</v>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 286.42 &lt;= EMA21 288.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>356</v>
+      </c>
+      <c r="E531" t="n">
+        <v>485.93</v>
+      </c>
+      <c r="F531" t="n">
+        <v>485.93</v>
+      </c>
+      <c r="G531" t="n">
+        <v>394.95</v>
+      </c>
+      <c r="H531" t="n">
+        <v>401.29</v>
+      </c>
+      <c r="I531" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J531" t="b">
+        <v>0</v>
+      </c>
+      <c r="K531" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 394.95 &lt;= EMA21 401.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>157.47</v>
+      </c>
+      <c r="E532" t="n">
+        <v>171.12</v>
+      </c>
+      <c r="F532" t="n">
+        <v>171.12</v>
+      </c>
+      <c r="G532" t="n">
+        <v>158.85</v>
+      </c>
+      <c r="H532" t="n">
+        <v>158.96</v>
+      </c>
+      <c r="I532" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J532" t="b">
+        <v>0</v>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 158.85 &lt;= EMA21 158.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D533" t="n">
+        <v>176.42</v>
+      </c>
+      <c r="E533" t="n">
+        <v>200.58</v>
+      </c>
+      <c r="F533" t="n">
+        <v>200.58</v>
+      </c>
+      <c r="G533" t="n">
+        <v>183.12</v>
+      </c>
+      <c r="H533" t="n">
+        <v>169.06</v>
+      </c>
+      <c r="I533" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J533" t="b">
+        <v>0</v>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 176.42 &lt;= Upper 200.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D534" t="n">
+        <v>186.28</v>
+      </c>
+      <c r="E534" t="n">
+        <v>211.25</v>
+      </c>
+      <c r="F534" t="n">
+        <v>211.25</v>
+      </c>
+      <c r="G534" t="n">
+        <v>196.09</v>
+      </c>
+      <c r="H534" t="n">
+        <v>190.64</v>
+      </c>
+      <c r="I534" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J534" t="b">
+        <v>0</v>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 186.28 &lt;= Upper 211.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D535" t="n">
+        <v>240.42</v>
+      </c>
+      <c r="E535" t="n">
+        <v>268.53</v>
+      </c>
+      <c r="F535" t="n">
+        <v>268.53</v>
+      </c>
+      <c r="G535" t="n">
+        <v>247.08</v>
+      </c>
+      <c r="H535" t="n">
+        <v>241.08</v>
+      </c>
+      <c r="I535" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J535" t="b">
+        <v>0</v>
+      </c>
+      <c r="K535" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 240.42 &lt;= Upper 268.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D536" t="n">
+        <v>264.84</v>
+      </c>
+      <c r="E536" t="n">
+        <v>293.84</v>
+      </c>
+      <c r="F536" t="n">
+        <v>293.84</v>
+      </c>
+      <c r="G536" t="n">
+        <v>271.07</v>
+      </c>
+      <c r="H536" t="n">
+        <v>256.75</v>
+      </c>
+      <c r="I536" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J536" t="b">
+        <v>0</v>
+      </c>
+      <c r="K536" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 264.84 &lt;= Upper 293.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D537" t="n">
+        <v>96.44</v>
+      </c>
+      <c r="E537" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="F537" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="G537" t="n">
+        <v>98.55</v>
+      </c>
+      <c r="H537" t="n">
+        <v>99.45</v>
+      </c>
+      <c r="I537" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J537" t="b">
+        <v>0</v>
+      </c>
+      <c r="K537" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 98.55 &lt;= EMA21 99.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D538" t="n">
+        <v>167.6</v>
+      </c>
+      <c r="E538" t="n">
+        <v>182.87</v>
+      </c>
+      <c r="F538" t="n">
+        <v>182.87</v>
+      </c>
+      <c r="G538" t="n">
+        <v>163.27</v>
+      </c>
+      <c r="H538" t="n">
+        <v>155.26</v>
+      </c>
+      <c r="I538" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J538" t="b">
+        <v>0</v>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 167.60 &lt;= Upper 182.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D539" t="n">
+        <v>312.01</v>
+      </c>
+      <c r="E539" t="n">
+        <v>322.36</v>
+      </c>
+      <c r="F539" t="n">
+        <v>322.36</v>
+      </c>
+      <c r="G539" t="n">
+        <v>314.71</v>
+      </c>
+      <c r="H539" t="n">
+        <v>326.93</v>
+      </c>
+      <c r="I539" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J539" t="b">
+        <v>0</v>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 314.71 &lt;= EMA21 326.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D540" t="n">
+        <v>505.43</v>
+      </c>
+      <c r="E540" t="n">
+        <v>678.45</v>
+      </c>
+      <c r="F540" t="n">
+        <v>678.45</v>
+      </c>
+      <c r="G540" t="n">
+        <v>543.5599999999999</v>
+      </c>
+      <c r="H540" t="n">
+        <v>564.23</v>
+      </c>
+      <c r="I540" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J540" t="b">
+        <v>0</v>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 543.56 &lt;= EMA21 564.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D541" t="n">
+        <v>284.11</v>
+      </c>
+      <c r="E541" t="n">
+        <v>350.94</v>
+      </c>
+      <c r="F541" t="n">
+        <v>350.94</v>
+      </c>
+      <c r="G541" t="n">
+        <v>308.87</v>
+      </c>
+      <c r="H541" t="n">
+        <v>319.92</v>
+      </c>
+      <c r="I541" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J541" t="b">
+        <v>0</v>
+      </c>
+      <c r="K541" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 308.87 &lt;= EMA21 319.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D542" t="n">
+        <v>392.03</v>
+      </c>
+      <c r="E542" t="n">
+        <v>449.41</v>
+      </c>
+      <c r="F542" t="n">
+        <v>449.41</v>
+      </c>
+      <c r="G542" t="n">
+        <v>410.71</v>
+      </c>
+      <c r="H542" t="n">
+        <v>411.95</v>
+      </c>
+      <c r="I542" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J542" t="b">
+        <v>0</v>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 410.71 &lt;= EMA21 411.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D543" t="n">
+        <v>212.21</v>
+      </c>
+      <c r="E543" t="n">
+        <v>275.03</v>
+      </c>
+      <c r="F543" t="n">
+        <v>275.03</v>
+      </c>
+      <c r="G543" t="n">
+        <v>236.89</v>
+      </c>
+      <c r="H543" t="n">
+        <v>241.83</v>
+      </c>
+      <c r="I543" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J543" t="b">
+        <v>0</v>
+      </c>
+      <c r="K543" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 236.89 &lt;= EMA21 241.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J544" t="b">
+        <v>0</v>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>133.26</v>
+      </c>
+      <c r="E545" t="n">
+        <v>162.12</v>
+      </c>
+      <c r="F545" t="n">
+        <v>162.12</v>
+      </c>
+      <c r="G545" t="n">
+        <v>146.68</v>
+      </c>
+      <c r="H545" t="n">
+        <v>147.05</v>
+      </c>
+      <c r="I545" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J545" t="b">
+        <v>0</v>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 146.68 &lt;= EMA21 147.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>347.82</v>
+      </c>
+      <c r="E546" t="n">
+        <v>391.79</v>
+      </c>
+      <c r="F546" t="n">
+        <v>391.79</v>
+      </c>
+      <c r="G546" t="n">
+        <v>362.98</v>
+      </c>
+      <c r="H546" t="n">
+        <v>351.67</v>
+      </c>
+      <c r="I546" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J546" t="b">
+        <v>0</v>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 347.82 &lt;= Upper 391.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>143.53</v>
+      </c>
+      <c r="E547" t="n">
+        <v>161.02</v>
+      </c>
+      <c r="F547" t="n">
+        <v>161.02</v>
+      </c>
+      <c r="G547" t="n">
+        <v>152.13</v>
+      </c>
+      <c r="H547" t="n">
+        <v>149.89</v>
+      </c>
+      <c r="I547" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J547" t="b">
+        <v>0</v>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 143.53 &lt;= Upper 161.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>172.59</v>
+      </c>
+      <c r="E548" t="n">
+        <v>205.53</v>
+      </c>
+      <c r="F548" t="n">
+        <v>205.53</v>
+      </c>
+      <c r="G548" t="n">
+        <v>187.82</v>
+      </c>
+      <c r="H548" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="I548" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J548" t="b">
+        <v>0</v>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 172.59 &lt;= Upper 205.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>59.92</v>
+      </c>
+      <c r="E549" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="F549" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="G549" t="n">
+        <v>62.37</v>
+      </c>
+      <c r="H549" t="n">
+        <v>60.46</v>
+      </c>
+      <c r="I549" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J549" t="b">
+        <v>0</v>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 59.92 &lt;= Upper 66.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="E550" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="F550" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="G550" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="H550" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="I550" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J550" t="b">
+        <v>0</v>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.78 &lt;= EMA21 11.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>115.31</v>
+      </c>
+      <c r="E551" t="n">
+        <v>123.66</v>
+      </c>
+      <c r="F551" t="n">
+        <v>123.66</v>
+      </c>
+      <c r="G551" t="n">
+        <v>115.14</v>
+      </c>
+      <c r="H551" t="n">
+        <v>110.39</v>
+      </c>
+      <c r="I551" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J551" t="b">
+        <v>0</v>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 115.31 &lt;= Upper 123.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>29.81</v>
+      </c>
+      <c r="E552" t="n">
+        <v>31.84</v>
+      </c>
+      <c r="F552" t="n">
+        <v>31.84</v>
+      </c>
+      <c r="G552" t="n">
+        <v>30.24</v>
+      </c>
+      <c r="H552" t="n">
+        <v>29.48</v>
+      </c>
+      <c r="I552" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J552" t="b">
+        <v>0</v>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 29.81 &lt;= Upper 31.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>144.48</v>
+      </c>
+      <c r="E553" t="n">
+        <v>156.47</v>
+      </c>
+      <c r="F553" t="n">
+        <v>156.47</v>
+      </c>
+      <c r="G553" t="n">
+        <v>147.55</v>
+      </c>
+      <c r="H553" t="n">
+        <v>144.07</v>
+      </c>
+      <c r="I553" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J553" t="b">
+        <v>0</v>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 144.48 &lt;= Upper 156.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>389.62</v>
+      </c>
+      <c r="E554" t="n">
+        <v>421.51</v>
+      </c>
+      <c r="F554" t="n">
+        <v>421.51</v>
+      </c>
+      <c r="G554" t="n">
+        <v>393.23</v>
+      </c>
+      <c r="H554" t="n">
+        <v>395.87</v>
+      </c>
+      <c r="I554" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J554" t="b">
+        <v>0</v>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 393.23 &lt;= EMA21 395.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J555" t="b">
+        <v>0</v>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>105.61</v>
+      </c>
+      <c r="E556" t="n">
+        <v>125.94</v>
+      </c>
+      <c r="F556" t="n">
+        <v>125.94</v>
+      </c>
+      <c r="G556" t="n">
+        <v>107.15</v>
+      </c>
+      <c r="H556" t="n">
+        <v>110.44</v>
+      </c>
+      <c r="I556" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J556" t="b">
+        <v>0</v>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.15 &lt;= EMA21 110.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J557" t="b">
+        <v>0</v>
+      </c>
+      <c r="K557" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>213.29</v>
+      </c>
+      <c r="E558" t="n">
+        <v>256.4</v>
+      </c>
+      <c r="F558" t="n">
+        <v>256.4</v>
+      </c>
+      <c r="G558" t="n">
+        <v>220.65</v>
+      </c>
+      <c r="H558" t="n">
+        <v>228.61</v>
+      </c>
+      <c r="I558" t="n">
+        <v>1</v>
+      </c>
+      <c r="J558" t="b">
+        <v>0</v>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 220.65 &lt;= EMA21 228.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D559" t="n">
+        <v>44.82</v>
+      </c>
+      <c r="E559" t="n">
+        <v>43.77</v>
+      </c>
+      <c r="F559" t="n">
+        <v>43.77</v>
+      </c>
+      <c r="G559" t="n">
+        <v>41.52</v>
+      </c>
+      <c r="H559" t="n">
+        <v>40.84</v>
+      </c>
+      <c r="I559" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J559" t="b">
+        <v>0</v>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.24x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="E560" t="n">
+        <v>48.45</v>
+      </c>
+      <c r="F560" t="n">
+        <v>48.45</v>
+      </c>
+      <c r="G560" t="n">
+        <v>42.55</v>
+      </c>
+      <c r="H560" t="n">
+        <v>42.07</v>
+      </c>
+      <c r="I560" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J560" t="b">
+        <v>0</v>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 42.75 &lt;= Upper 48.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>76.77</v>
+      </c>
+      <c r="E561" t="n">
+        <v>84.34</v>
+      </c>
+      <c r="F561" t="n">
+        <v>84.34</v>
+      </c>
+      <c r="G561" t="n">
+        <v>79.84999999999999</v>
+      </c>
+      <c r="H561" t="n">
+        <v>78.91</v>
+      </c>
+      <c r="I561" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J561" t="b">
+        <v>0</v>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 76.77 &lt;= Upper 84.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>105.06</v>
+      </c>
+      <c r="E562" t="n">
+        <v>111.25</v>
+      </c>
+      <c r="F562" t="n">
+        <v>111.25</v>
+      </c>
+      <c r="G562" t="n">
+        <v>106.63</v>
+      </c>
+      <c r="H562" t="n">
+        <v>105.77</v>
+      </c>
+      <c r="I562" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J562" t="b">
+        <v>0</v>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 105.06 &lt;= Upper 111.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>28.12</v>
+      </c>
+      <c r="E563" t="n">
+        <v>29.23</v>
+      </c>
+      <c r="F563" t="n">
+        <v>29.23</v>
+      </c>
+      <c r="G563" t="n">
+        <v>28.35</v>
+      </c>
+      <c r="H563" t="n">
+        <v>28.07</v>
+      </c>
+      <c r="I563" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J563" t="b">
+        <v>0</v>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 28.12 &lt;= Upper 29.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E564" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F564" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G564" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="H564" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="I564" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J564" t="b">
+        <v>0</v>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1.11 &lt;= EMA21 1.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>528.64</v>
+      </c>
+      <c r="E565" t="n">
+        <v>573.75</v>
+      </c>
+      <c r="F565" t="n">
+        <v>573.75</v>
+      </c>
+      <c r="G565" t="n">
+        <v>541.74</v>
+      </c>
+      <c r="H565" t="n">
+        <v>530.77</v>
+      </c>
+      <c r="I565" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J565" t="b">
+        <v>0</v>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 528.64 &lt;= Upper 573.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D566" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="E566" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="F566" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="G566" t="n">
+        <v>8.359999999999999</v>
+      </c>
+      <c r="H566" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="I566" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J566" t="b">
+        <v>0</v>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8.36 &lt;= EMA21 8.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>106.05</v>
+      </c>
+      <c r="E567" t="n">
+        <v>118.13</v>
+      </c>
+      <c r="F567" t="n">
+        <v>118.13</v>
+      </c>
+      <c r="G567" t="n">
+        <v>106.44</v>
+      </c>
+      <c r="H567" t="n">
+        <v>107.81</v>
+      </c>
+      <c r="I567" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J567" t="b">
+        <v>0</v>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.44 &lt;= EMA21 107.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D568" t="n">
+        <v>910.1799999999999</v>
+      </c>
+      <c r="E568" t="n">
+        <v>977.8099999999999</v>
+      </c>
+      <c r="F568" t="n">
+        <v>977.8099999999999</v>
+      </c>
+      <c r="G568" t="n">
+        <v>930.0599999999999</v>
+      </c>
+      <c r="H568" t="n">
+        <v>939.61</v>
+      </c>
+      <c r="I568" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J568" t="b">
+        <v>0</v>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 930.06 &lt;= EMA21 939.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>162.71</v>
+      </c>
+      <c r="E569" t="n">
+        <v>171.35</v>
+      </c>
+      <c r="F569" t="n">
+        <v>171.35</v>
+      </c>
+      <c r="G569" t="n">
+        <v>163</v>
+      </c>
+      <c r="H569" t="n">
+        <v>159.15</v>
+      </c>
+      <c r="I569" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J569" t="b">
+        <v>0</v>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 162.71 &lt;= Upper 171.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>313.7</v>
+      </c>
+      <c r="E570" t="n">
+        <v>350.5</v>
+      </c>
+      <c r="F570" t="n">
+        <v>350.5</v>
+      </c>
+      <c r="G570" t="n">
+        <v>321.73</v>
+      </c>
+      <c r="H570" t="n">
+        <v>328.04</v>
+      </c>
+      <c r="I570" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J570" t="b">
+        <v>0</v>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 321.73 &lt;= EMA21 328.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>200.8</v>
+      </c>
+      <c r="E571" t="n">
+        <v>225.99</v>
+      </c>
+      <c r="F571" t="n">
+        <v>225.99</v>
+      </c>
+      <c r="G571" t="n">
+        <v>204.7</v>
+      </c>
+      <c r="H571" t="n">
+        <v>208.84</v>
+      </c>
+      <c r="I571" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J571" t="b">
+        <v>0</v>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 204.70 &lt;= EMA21 208.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="E572" t="n">
+        <v>59.42</v>
+      </c>
+      <c r="F572" t="n">
+        <v>59.42</v>
+      </c>
+      <c r="G572" t="n">
+        <v>57.87</v>
+      </c>
+      <c r="H572" t="n">
+        <v>57.64</v>
+      </c>
+      <c r="I572" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J572" t="b">
+        <v>0</v>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 57.20 &lt;= Upper 59.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="E573" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="F573" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="G573" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="H573" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="I573" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J573" t="b">
+        <v>0</v>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12.39 &lt;= EMA21 12.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>127.87</v>
+      </c>
+      <c r="E574" t="n">
+        <v>133.09</v>
+      </c>
+      <c r="F574" t="n">
+        <v>133.09</v>
+      </c>
+      <c r="G574" t="n">
+        <v>128.46</v>
+      </c>
+      <c r="H574" t="n">
+        <v>126.14</v>
+      </c>
+      <c r="I574" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J574" t="b">
+        <v>0</v>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 127.87 &lt;= Upper 133.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>124.04</v>
+      </c>
+      <c r="E575" t="n">
+        <v>135.82</v>
+      </c>
+      <c r="F575" t="n">
+        <v>135.82</v>
+      </c>
+      <c r="G575" t="n">
+        <v>129.4</v>
+      </c>
+      <c r="H575" t="n">
+        <v>129.42</v>
+      </c>
+      <c r="I575" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J575" t="b">
+        <v>0</v>
+      </c>
+      <c r="K575" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 129.40 &lt;= EMA21 129.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>89.84999999999999</v>
+      </c>
+      <c r="E576" t="n">
+        <v>97.08</v>
+      </c>
+      <c r="F576" t="n">
+        <v>97.08</v>
+      </c>
+      <c r="G576" t="n">
+        <v>92.13</v>
+      </c>
+      <c r="H576" t="n">
+        <v>92.84999999999999</v>
+      </c>
+      <c r="I576" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J576" t="b">
+        <v>0</v>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 92.13 &lt;= EMA21 92.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>229.31</v>
+      </c>
+      <c r="E577" t="n">
+        <v>250.62</v>
+      </c>
+      <c r="F577" t="n">
+        <v>250.62</v>
+      </c>
+      <c r="G577" t="n">
+        <v>231.61</v>
+      </c>
+      <c r="H577" t="n">
+        <v>235.01</v>
+      </c>
+      <c r="I577" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J577" t="b">
+        <v>0</v>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 231.61 &lt;= EMA21 235.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>128.92</v>
+      </c>
+      <c r="E578" t="n">
+        <v>158.28</v>
+      </c>
+      <c r="F578" t="n">
+        <v>158.28</v>
+      </c>
+      <c r="G578" t="n">
+        <v>133.75</v>
+      </c>
+      <c r="H578" t="n">
+        <v>139.88</v>
+      </c>
+      <c r="I578" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J578" t="b">
+        <v>0</v>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 133.75 &lt;= EMA21 139.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="E579" t="n">
+        <v>41.33</v>
+      </c>
+      <c r="F579" t="n">
+        <v>41.33</v>
+      </c>
+      <c r="G579" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="H579" t="n">
+        <v>39.37</v>
+      </c>
+      <c r="I579" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J579" t="b">
+        <v>0</v>
+      </c>
+      <c r="K579" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 38.60 &lt;= EMA21 39.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>103.19</v>
+      </c>
+      <c r="E580" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="F580" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="G580" t="n">
+        <v>113.32</v>
+      </c>
+      <c r="H580" t="n">
+        <v>116.57</v>
+      </c>
+      <c r="I580" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="J580" t="b">
+        <v>0</v>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 113.32 &lt;= EMA21 116.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>102.01</v>
+      </c>
+      <c r="E581" t="n">
+        <v>109.61</v>
+      </c>
+      <c r="F581" t="n">
+        <v>109.61</v>
+      </c>
+      <c r="G581" t="n">
+        <v>105.29</v>
+      </c>
+      <c r="H581" t="n">
+        <v>105.66</v>
+      </c>
+      <c r="I581" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J581" t="b">
+        <v>0</v>
+      </c>
+      <c r="K581" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 105.29 &lt;= EMA21 105.66)</t>
         </is>
       </c>
     </row>
@@ -20926,7 +25172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21147,6 +25393,99 @@
         <v>1.34</v>
       </c>
       <c r="G7" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="E8" t="n">
+        <v>155.21</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="E9" t="n">
+        <v>166.26</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>99.39</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -21163,7 +25502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21259,6 +25598,129 @@
         <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1914.99</v>
+      </c>
+      <c r="F3" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>166.26</v>
+      </c>
+      <c r="I3" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1950.24</v>
+      </c>
+      <c r="F4" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>155.21</v>
+      </c>
+      <c r="I4" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1977.33</v>
+      </c>
+      <c r="F5" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>99.39</v>
+      </c>
+      <c r="I5" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -21458,7 +25920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21709,6 +26171,153 @@
         </is>
       </c>
       <c r="K5" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-09 04:53:26</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>83C0264FA2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="G6" t="n">
+        <v>174.09</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-09 04:53:26</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>14C96CCE2E</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="G7" t="n">
+        <v>162.52</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>12</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-09 04:53:26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BCEF2D0EB1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="G8" t="n">
+        <v>104.07</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>19</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
         </is>
@@ -21793,7 +26402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22140,6 +26749,39 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:53:28</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2413.74</v>
+      </c>
+      <c r="D11" t="n">
+        <v>7414.98</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-171.28</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-10T04:43 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K581"/>
+  <dimension ref="A1:K681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25158,6 +25158,4252 @@
       <c r="K581" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 105.29 &lt;= EMA21 105.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>315.34</v>
+      </c>
+      <c r="E582" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="F582" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="G582" t="n">
+        <v>318.45</v>
+      </c>
+      <c r="H582" t="n">
+        <v>316.56</v>
+      </c>
+      <c r="I582" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J582" t="b">
+        <v>0</v>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 315.34 &lt;= Upper 328.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>491.65</v>
+      </c>
+      <c r="E583" t="n">
+        <v>514.12</v>
+      </c>
+      <c r="F583" t="n">
+        <v>514.12</v>
+      </c>
+      <c r="G583" t="n">
+        <v>497.67</v>
+      </c>
+      <c r="H583" t="n">
+        <v>489.39</v>
+      </c>
+      <c r="I583" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J583" t="b">
+        <v>0</v>
+      </c>
+      <c r="K583" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 491.65 &lt;= Upper 514.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>223.67</v>
+      </c>
+      <c r="E584" t="n">
+        <v>233.25</v>
+      </c>
+      <c r="F584" t="n">
+        <v>233.25</v>
+      </c>
+      <c r="G584" t="n">
+        <v>223.5</v>
+      </c>
+      <c r="H584" t="n">
+        <v>220.01</v>
+      </c>
+      <c r="I584" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J584" t="b">
+        <v>0</v>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 223.67 &lt;= Upper 233.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>330.65</v>
+      </c>
+      <c r="E585" t="n">
+        <v>350.67</v>
+      </c>
+      <c r="F585" t="n">
+        <v>350.67</v>
+      </c>
+      <c r="G585" t="n">
+        <v>338.24</v>
+      </c>
+      <c r="H585" t="n">
+        <v>341.81</v>
+      </c>
+      <c r="I585" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J585" t="b">
+        <v>0</v>
+      </c>
+      <c r="K585" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 338.24 &lt;= EMA21 341.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>328.38</v>
+      </c>
+      <c r="E586" t="n">
+        <v>347.7</v>
+      </c>
+      <c r="F586" t="n">
+        <v>347.7</v>
+      </c>
+      <c r="G586" t="n">
+        <v>335.24</v>
+      </c>
+      <c r="H586" t="n">
+        <v>339.05</v>
+      </c>
+      <c r="I586" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J586" t="b">
+        <v>0</v>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 335.24 &lt;= EMA21 339.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>252.4</v>
+      </c>
+      <c r="E587" t="n">
+        <v>268.18</v>
+      </c>
+      <c r="F587" t="n">
+        <v>268.18</v>
+      </c>
+      <c r="G587" t="n">
+        <v>257.33</v>
+      </c>
+      <c r="H587" t="n">
+        <v>258.68</v>
+      </c>
+      <c r="I587" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J587" t="b">
+        <v>0</v>
+      </c>
+      <c r="K587" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 257.33 &lt;= EMA21 258.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>653.6900000000001</v>
+      </c>
+      <c r="E588" t="n">
+        <v>636.16</v>
+      </c>
+      <c r="F588" t="n">
+        <v>636.16</v>
+      </c>
+      <c r="G588" t="n">
+        <v>606.27</v>
+      </c>
+      <c r="H588" t="n">
+        <v>592.4400000000001</v>
+      </c>
+      <c r="I588" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="J588" t="b">
+        <v>1</v>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>367.81</v>
+      </c>
+      <c r="E589" t="n">
+        <v>376.63</v>
+      </c>
+      <c r="F589" t="n">
+        <v>376.63</v>
+      </c>
+      <c r="G589" t="n">
+        <v>361.17</v>
+      </c>
+      <c r="H589" t="n">
+        <v>354.5</v>
+      </c>
+      <c r="I589" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J589" t="b">
+        <v>0</v>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 367.81 &lt;= Upper 376.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>364.38</v>
+      </c>
+      <c r="E590" t="n">
+        <v>409.51</v>
+      </c>
+      <c r="F590" t="n">
+        <v>409.51</v>
+      </c>
+      <c r="G590" t="n">
+        <v>365.62</v>
+      </c>
+      <c r="H590" t="n">
+        <v>372.78</v>
+      </c>
+      <c r="I590" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J590" t="b">
+        <v>0</v>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.62 &lt;= EMA21 372.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>161.63</v>
+      </c>
+      <c r="E591" t="n">
+        <v>162.63</v>
+      </c>
+      <c r="F591" t="n">
+        <v>162.63</v>
+      </c>
+      <c r="G591" t="n">
+        <v>154.41</v>
+      </c>
+      <c r="H591" t="n">
+        <v>149.71</v>
+      </c>
+      <c r="I591" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J591" t="b">
+        <v>0</v>
+      </c>
+      <c r="K591" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 161.63 &lt;= Upper 162.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>244.16</v>
+      </c>
+      <c r="E592" t="n">
+        <v>281.85</v>
+      </c>
+      <c r="F592" t="n">
+        <v>281.85</v>
+      </c>
+      <c r="G592" t="n">
+        <v>246.9</v>
+      </c>
+      <c r="H592" t="n">
+        <v>229.7</v>
+      </c>
+      <c r="I592" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J592" t="b">
+        <v>0</v>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 244.16 &lt;= Upper 281.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>254.86</v>
+      </c>
+      <c r="E593" t="n">
+        <v>296.99</v>
+      </c>
+      <c r="F593" t="n">
+        <v>296.99</v>
+      </c>
+      <c r="G593" t="n">
+        <v>270.78</v>
+      </c>
+      <c r="H593" t="n">
+        <v>269.53</v>
+      </c>
+      <c r="I593" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J593" t="b">
+        <v>0</v>
+      </c>
+      <c r="K593" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 254.86 &lt;= Upper 296.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>521.09</v>
+      </c>
+      <c r="E594" t="n">
+        <v>517.58</v>
+      </c>
+      <c r="F594" t="n">
+        <v>517.58</v>
+      </c>
+      <c r="G594" t="n">
+        <v>484.84</v>
+      </c>
+      <c r="H594" t="n">
+        <v>482.15</v>
+      </c>
+      <c r="I594" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J594" t="b">
+        <v>0</v>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.22x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>106.24</v>
+      </c>
+      <c r="E595" t="n">
+        <v>107.81</v>
+      </c>
+      <c r="F595" t="n">
+        <v>107.81</v>
+      </c>
+      <c r="G595" t="n">
+        <v>96.69</v>
+      </c>
+      <c r="H595" t="n">
+        <v>95.53</v>
+      </c>
+      <c r="I595" t="n">
+        <v>1</v>
+      </c>
+      <c r="J595" t="b">
+        <v>0</v>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 106.24 &lt;= Upper 107.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>1027.77</v>
+      </c>
+      <c r="E596" t="n">
+        <v>1025.53</v>
+      </c>
+      <c r="F596" t="n">
+        <v>1025.53</v>
+      </c>
+      <c r="G596" t="n">
+        <v>980</v>
+      </c>
+      <c r="H596" t="n">
+        <v>955.9</v>
+      </c>
+      <c r="I596" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J596" t="b">
+        <v>0</v>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.86x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="E597" t="n">
+        <v>174.73</v>
+      </c>
+      <c r="F597" t="n">
+        <v>174.73</v>
+      </c>
+      <c r="G597" t="n">
+        <v>169.51</v>
+      </c>
+      <c r="H597" t="n">
+        <v>166.72</v>
+      </c>
+      <c r="I597" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J597" t="b">
+        <v>1</v>
+      </c>
+      <c r="K597" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>261.59</v>
+      </c>
+      <c r="E598" t="n">
+        <v>281.54</v>
+      </c>
+      <c r="F598" t="n">
+        <v>281.54</v>
+      </c>
+      <c r="G598" t="n">
+        <v>259.51</v>
+      </c>
+      <c r="H598" t="n">
+        <v>264.55</v>
+      </c>
+      <c r="I598" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J598" t="b">
+        <v>0</v>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 259.51 &lt;= EMA21 264.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>468.85</v>
+      </c>
+      <c r="E599" t="n">
+        <v>547.95</v>
+      </c>
+      <c r="F599" t="n">
+        <v>547.95</v>
+      </c>
+      <c r="G599" t="n">
+        <v>463.27</v>
+      </c>
+      <c r="H599" t="n">
+        <v>480.28</v>
+      </c>
+      <c r="I599" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J599" t="b">
+        <v>0</v>
+      </c>
+      <c r="K599" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 463.27 &lt;= EMA21 480.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>315.84</v>
+      </c>
+      <c r="E600" t="n">
+        <v>343.63</v>
+      </c>
+      <c r="F600" t="n">
+        <v>343.63</v>
+      </c>
+      <c r="G600" t="n">
+        <v>307.92</v>
+      </c>
+      <c r="H600" t="n">
+        <v>309.83</v>
+      </c>
+      <c r="I600" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J600" t="b">
+        <v>0</v>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 307.92 &lt;= EMA21 309.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>182.91</v>
+      </c>
+      <c r="E601" t="n">
+        <v>210.39</v>
+      </c>
+      <c r="F601" t="n">
+        <v>210.39</v>
+      </c>
+      <c r="G601" t="n">
+        <v>181.58</v>
+      </c>
+      <c r="H601" t="n">
+        <v>185.82</v>
+      </c>
+      <c r="I601" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J601" t="b">
+        <v>0</v>
+      </c>
+      <c r="K601" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 181.58 &lt;= EMA21 185.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>1729.52</v>
+      </c>
+      <c r="E602" t="n">
+        <v>1874.99</v>
+      </c>
+      <c r="F602" t="n">
+        <v>1874.99</v>
+      </c>
+      <c r="G602" t="n">
+        <v>1717.98</v>
+      </c>
+      <c r="H602" t="n">
+        <v>1728.15</v>
+      </c>
+      <c r="I602" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J602" t="b">
+        <v>0</v>
+      </c>
+      <c r="K602" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1717.98 &lt;= EMA21 1728.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>365.07</v>
+      </c>
+      <c r="E603" t="n">
+        <v>390.02</v>
+      </c>
+      <c r="F603" t="n">
+        <v>390.02</v>
+      </c>
+      <c r="G603" t="n">
+        <v>363.13</v>
+      </c>
+      <c r="H603" t="n">
+        <v>367.66</v>
+      </c>
+      <c r="I603" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J603" t="b">
+        <v>0</v>
+      </c>
+      <c r="K603" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.13 &lt;= EMA21 367.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>235.01</v>
+      </c>
+      <c r="E604" t="n">
+        <v>252.79</v>
+      </c>
+      <c r="F604" t="n">
+        <v>252.79</v>
+      </c>
+      <c r="G604" t="n">
+        <v>223.49</v>
+      </c>
+      <c r="H604" t="n">
+        <v>222.55</v>
+      </c>
+      <c r="I604" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J604" t="b">
+        <v>0</v>
+      </c>
+      <c r="K604" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 235.01 &lt;= Upper 252.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>223.32</v>
+      </c>
+      <c r="E605" t="n">
+        <v>234.32</v>
+      </c>
+      <c r="F605" t="n">
+        <v>234.32</v>
+      </c>
+      <c r="G605" t="n">
+        <v>225.13</v>
+      </c>
+      <c r="H605" t="n">
+        <v>229.34</v>
+      </c>
+      <c r="I605" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J605" t="b">
+        <v>0</v>
+      </c>
+      <c r="K605" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 225.13 &lt;= EMA21 229.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>70.98</v>
+      </c>
+      <c r="E606" t="n">
+        <v>83.84999999999999</v>
+      </c>
+      <c r="F606" t="n">
+        <v>83.84999999999999</v>
+      </c>
+      <c r="G606" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="H606" t="n">
+        <v>75.62</v>
+      </c>
+      <c r="I606" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J606" t="b">
+        <v>0</v>
+      </c>
+      <c r="K606" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 72.90 &lt;= EMA21 75.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>1203.75</v>
+      </c>
+      <c r="E607" t="n">
+        <v>1431.71</v>
+      </c>
+      <c r="F607" t="n">
+        <v>1431.71</v>
+      </c>
+      <c r="G607" t="n">
+        <v>1237.52</v>
+      </c>
+      <c r="H607" t="n">
+        <v>1278.16</v>
+      </c>
+      <c r="I607" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J607" t="b">
+        <v>0</v>
+      </c>
+      <c r="K607" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1237.52 &lt;= EMA21 1278.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>76.54000000000001</v>
+      </c>
+      <c r="E608" t="n">
+        <v>75.45</v>
+      </c>
+      <c r="F608" t="n">
+        <v>75.45</v>
+      </c>
+      <c r="G608" t="n">
+        <v>72</v>
+      </c>
+      <c r="H608" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="I608" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J608" t="b">
+        <v>0</v>
+      </c>
+      <c r="K608" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.83x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>105.24</v>
+      </c>
+      <c r="E609" t="n">
+        <v>104.21</v>
+      </c>
+      <c r="F609" t="n">
+        <v>104.21</v>
+      </c>
+      <c r="G609" t="n">
+        <v>100.77</v>
+      </c>
+      <c r="H609" t="n">
+        <v>98.05</v>
+      </c>
+      <c r="I609" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J609" t="b">
+        <v>0</v>
+      </c>
+      <c r="K609" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.04x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D610" t="n">
+        <v>383.69</v>
+      </c>
+      <c r="E610" t="n">
+        <v>432.48</v>
+      </c>
+      <c r="F610" t="n">
+        <v>432.48</v>
+      </c>
+      <c r="G610" t="n">
+        <v>363.02</v>
+      </c>
+      <c r="H610" t="n">
+        <v>367.12</v>
+      </c>
+      <c r="I610" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J610" t="b">
+        <v>0</v>
+      </c>
+      <c r="K610" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.02 &lt;= EMA21 367.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D611" t="n">
+        <v>143.03</v>
+      </c>
+      <c r="E611" t="n">
+        <v>165.68</v>
+      </c>
+      <c r="F611" t="n">
+        <v>165.68</v>
+      </c>
+      <c r="G611" t="n">
+        <v>138.59</v>
+      </c>
+      <c r="H611" t="n">
+        <v>140.13</v>
+      </c>
+      <c r="I611" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J611" t="b">
+        <v>0</v>
+      </c>
+      <c r="K611" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 138.59 &lt;= EMA21 140.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D612" t="n">
+        <v>73.01000000000001</v>
+      </c>
+      <c r="E612" t="n">
+        <v>79.81999999999999</v>
+      </c>
+      <c r="F612" t="n">
+        <v>79.81999999999999</v>
+      </c>
+      <c r="G612" t="n">
+        <v>73.56</v>
+      </c>
+      <c r="H612" t="n">
+        <v>75.02</v>
+      </c>
+      <c r="I612" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J612" t="b">
+        <v>0</v>
+      </c>
+      <c r="K612" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 73.56 &lt;= EMA21 75.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D613" t="n">
+        <v>38.93</v>
+      </c>
+      <c r="E613" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="F613" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="G613" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="H613" t="n">
+        <v>36.77</v>
+      </c>
+      <c r="I613" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J613" t="b">
+        <v>0</v>
+      </c>
+      <c r="K613" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 38.93 &lt;= Upper 40.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D614" t="n">
+        <v>535.25</v>
+      </c>
+      <c r="E614" t="n">
+        <v>542.76</v>
+      </c>
+      <c r="F614" t="n">
+        <v>542.76</v>
+      </c>
+      <c r="G614" t="n">
+        <v>500.27</v>
+      </c>
+      <c r="H614" t="n">
+        <v>476.53</v>
+      </c>
+      <c r="I614" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J614" t="b">
+        <v>0</v>
+      </c>
+      <c r="K614" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 535.25 &lt;= Upper 542.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D615" t="n">
+        <v>32.39</v>
+      </c>
+      <c r="E615" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="F615" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="G615" t="n">
+        <v>31.41</v>
+      </c>
+      <c r="H615" t="n">
+        <v>30.36</v>
+      </c>
+      <c r="I615" t="n">
+        <v>1</v>
+      </c>
+      <c r="J615" t="b">
+        <v>0</v>
+      </c>
+      <c r="K615" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 32.39 &lt;= Upper 32.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D616" t="n">
+        <v>482.28</v>
+      </c>
+      <c r="E616" t="n">
+        <v>516.8</v>
+      </c>
+      <c r="F616" t="n">
+        <v>516.8</v>
+      </c>
+      <c r="G616" t="n">
+        <v>465.08</v>
+      </c>
+      <c r="H616" t="n">
+        <v>470.42</v>
+      </c>
+      <c r="I616" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J616" t="b">
+        <v>0</v>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 465.08 &lt;= EMA21 470.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D617" t="n">
+        <v>885.92</v>
+      </c>
+      <c r="E617" t="n">
+        <v>971.3099999999999</v>
+      </c>
+      <c r="F617" t="n">
+        <v>971.3099999999999</v>
+      </c>
+      <c r="G617" t="n">
+        <v>852.87</v>
+      </c>
+      <c r="H617" t="n">
+        <v>850.46</v>
+      </c>
+      <c r="I617" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J617" t="b">
+        <v>0</v>
+      </c>
+      <c r="K617" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 885.92 &lt;= Upper 971.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>192.93</v>
+      </c>
+      <c r="E618" t="n">
+        <v>208.18</v>
+      </c>
+      <c r="F618" t="n">
+        <v>208.18</v>
+      </c>
+      <c r="G618" t="n">
+        <v>192.96</v>
+      </c>
+      <c r="H618" t="n">
+        <v>191.69</v>
+      </c>
+      <c r="I618" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J618" t="b">
+        <v>0</v>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 192.93 &lt;= Upper 208.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>109.43</v>
+      </c>
+      <c r="E619" t="n">
+        <v>117.82</v>
+      </c>
+      <c r="F619" t="n">
+        <v>117.82</v>
+      </c>
+      <c r="G619" t="n">
+        <v>109.85</v>
+      </c>
+      <c r="H619" t="n">
+        <v>111.47</v>
+      </c>
+      <c r="I619" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J619" t="b">
+        <v>0</v>
+      </c>
+      <c r="K619" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.85 &lt;= EMA21 111.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>175.8</v>
+      </c>
+      <c r="E620" t="n">
+        <v>195.29</v>
+      </c>
+      <c r="F620" t="n">
+        <v>195.29</v>
+      </c>
+      <c r="G620" t="n">
+        <v>183.72</v>
+      </c>
+      <c r="H620" t="n">
+        <v>180.77</v>
+      </c>
+      <c r="I620" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J620" t="b">
+        <v>0</v>
+      </c>
+      <c r="K620" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 175.80 &lt;= Upper 195.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>239.94</v>
+      </c>
+      <c r="E621" t="n">
+        <v>239.95</v>
+      </c>
+      <c r="F621" t="n">
+        <v>239.95</v>
+      </c>
+      <c r="G621" t="n">
+        <v>234.78</v>
+      </c>
+      <c r="H621" t="n">
+        <v>234.24</v>
+      </c>
+      <c r="I621" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J621" t="b">
+        <v>0</v>
+      </c>
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 239.94 &lt;= Upper 239.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>131.11</v>
+      </c>
+      <c r="E622" t="n">
+        <v>149.85</v>
+      </c>
+      <c r="F622" t="n">
+        <v>149.85</v>
+      </c>
+      <c r="G622" t="n">
+        <v>136.6</v>
+      </c>
+      <c r="H622" t="n">
+        <v>131.86</v>
+      </c>
+      <c r="I622" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J622" t="b">
+        <v>0</v>
+      </c>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 131.11 &lt;= Upper 149.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>313.94</v>
+      </c>
+      <c r="E623" t="n">
+        <v>377.7</v>
+      </c>
+      <c r="F623" t="n">
+        <v>377.7</v>
+      </c>
+      <c r="G623" t="n">
+        <v>335.33</v>
+      </c>
+      <c r="H623" t="n">
+        <v>338.25</v>
+      </c>
+      <c r="I623" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J623" t="b">
+        <v>0</v>
+      </c>
+      <c r="K623" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 335.33 &lt;= EMA21 338.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>335.1</v>
+      </c>
+      <c r="E624" t="n">
+        <v>402.15</v>
+      </c>
+      <c r="F624" t="n">
+        <v>402.15</v>
+      </c>
+      <c r="G624" t="n">
+        <v>344.25</v>
+      </c>
+      <c r="H624" t="n">
+        <v>350.74</v>
+      </c>
+      <c r="I624" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J624" t="b">
+        <v>0</v>
+      </c>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 344.25 &lt;= EMA21 350.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>207.8</v>
+      </c>
+      <c r="E625" t="n">
+        <v>236.53</v>
+      </c>
+      <c r="F625" t="n">
+        <v>236.53</v>
+      </c>
+      <c r="G625" t="n">
+        <v>210.52</v>
+      </c>
+      <c r="H625" t="n">
+        <v>208.25</v>
+      </c>
+      <c r="I625" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J625" t="b">
+        <v>0</v>
+      </c>
+      <c r="K625" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 207.80 &lt;= Upper 236.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>331.48</v>
+      </c>
+      <c r="E626" t="n">
+        <v>348.86</v>
+      </c>
+      <c r="F626" t="n">
+        <v>348.86</v>
+      </c>
+      <c r="G626" t="n">
+        <v>331.07</v>
+      </c>
+      <c r="H626" t="n">
+        <v>324.33</v>
+      </c>
+      <c r="I626" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J626" t="b">
+        <v>0</v>
+      </c>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 331.48 &lt;= Upper 348.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>169.53</v>
+      </c>
+      <c r="E627" t="n">
+        <v>187.54</v>
+      </c>
+      <c r="F627" t="n">
+        <v>187.54</v>
+      </c>
+      <c r="G627" t="n">
+        <v>175</v>
+      </c>
+      <c r="H627" t="n">
+        <v>171.6</v>
+      </c>
+      <c r="I627" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J627" t="b">
+        <v>0</v>
+      </c>
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.53 &lt;= Upper 187.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>225.27</v>
+      </c>
+      <c r="E628" t="n">
+        <v>259.03</v>
+      </c>
+      <c r="F628" t="n">
+        <v>259.03</v>
+      </c>
+      <c r="G628" t="n">
+        <v>221.72</v>
+      </c>
+      <c r="H628" t="n">
+        <v>230.6</v>
+      </c>
+      <c r="I628" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J628" t="b">
+        <v>0</v>
+      </c>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 221.72 &lt;= EMA21 230.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>166.1</v>
+      </c>
+      <c r="E629" t="n">
+        <v>193.9</v>
+      </c>
+      <c r="F629" t="n">
+        <v>193.9</v>
+      </c>
+      <c r="G629" t="n">
+        <v>172.33</v>
+      </c>
+      <c r="H629" t="n">
+        <v>172.75</v>
+      </c>
+      <c r="I629" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J629" t="b">
+        <v>0</v>
+      </c>
+      <c r="K629" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 172.33 &lt;= EMA21 172.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>314.18</v>
+      </c>
+      <c r="E630" t="n">
+        <v>327.11</v>
+      </c>
+      <c r="F630" t="n">
+        <v>327.11</v>
+      </c>
+      <c r="G630" t="n">
+        <v>291.97</v>
+      </c>
+      <c r="H630" t="n">
+        <v>290.9</v>
+      </c>
+      <c r="I630" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J630" t="b">
+        <v>0</v>
+      </c>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 314.18 &lt;= Upper 327.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>358.38</v>
+      </c>
+      <c r="E631" t="n">
+        <v>487.43</v>
+      </c>
+      <c r="F631" t="n">
+        <v>487.43</v>
+      </c>
+      <c r="G631" t="n">
+        <v>387.64</v>
+      </c>
+      <c r="H631" t="n">
+        <v>397.39</v>
+      </c>
+      <c r="I631" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J631" t="b">
+        <v>0</v>
+      </c>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 387.64 &lt;= EMA21 397.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>157.22</v>
+      </c>
+      <c r="E632" t="n">
+        <v>170.83</v>
+      </c>
+      <c r="F632" t="n">
+        <v>170.83</v>
+      </c>
+      <c r="G632" t="n">
+        <v>158.52</v>
+      </c>
+      <c r="H632" t="n">
+        <v>158.8</v>
+      </c>
+      <c r="I632" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J632" t="b">
+        <v>0</v>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 158.52 &lt;= EMA21 158.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>177.74</v>
+      </c>
+      <c r="E633" t="n">
+        <v>199.94</v>
+      </c>
+      <c r="F633" t="n">
+        <v>199.94</v>
+      </c>
+      <c r="G633" t="n">
+        <v>182.05</v>
+      </c>
+      <c r="H633" t="n">
+        <v>169.85</v>
+      </c>
+      <c r="I633" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J633" t="b">
+        <v>0</v>
+      </c>
+      <c r="K633" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 177.74 &lt;= Upper 199.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>186.05</v>
+      </c>
+      <c r="E634" t="n">
+        <v>210.72</v>
+      </c>
+      <c r="F634" t="n">
+        <v>210.72</v>
+      </c>
+      <c r="G634" t="n">
+        <v>194.08</v>
+      </c>
+      <c r="H634" t="n">
+        <v>190.22</v>
+      </c>
+      <c r="I634" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J634" t="b">
+        <v>0</v>
+      </c>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 186.05 &lt;= Upper 210.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>230.19</v>
+      </c>
+      <c r="E635" t="n">
+        <v>267.96</v>
+      </c>
+      <c r="F635" t="n">
+        <v>267.96</v>
+      </c>
+      <c r="G635" t="n">
+        <v>243.7</v>
+      </c>
+      <c r="H635" t="n">
+        <v>240.09</v>
+      </c>
+      <c r="I635" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J635" t="b">
+        <v>0</v>
+      </c>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 230.19 &lt;= Upper 267.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>260.8</v>
+      </c>
+      <c r="E636" t="n">
+        <v>293.48</v>
+      </c>
+      <c r="F636" t="n">
+        <v>293.48</v>
+      </c>
+      <c r="G636" t="n">
+        <v>269.02</v>
+      </c>
+      <c r="H636" t="n">
+        <v>257.11</v>
+      </c>
+      <c r="I636" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J636" t="b">
+        <v>0</v>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 260.80 &lt;= Upper 293.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>96.18000000000001</v>
+      </c>
+      <c r="E637" t="n">
+        <v>111.44</v>
+      </c>
+      <c r="F637" t="n">
+        <v>111.44</v>
+      </c>
+      <c r="G637" t="n">
+        <v>98.06999999999999</v>
+      </c>
+      <c r="H637" t="n">
+        <v>99.15000000000001</v>
+      </c>
+      <c r="I637" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J637" t="b">
+        <v>0</v>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 98.07 &lt;= EMA21 99.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>172.74</v>
+      </c>
+      <c r="E638" t="n">
+        <v>185.31</v>
+      </c>
+      <c r="F638" t="n">
+        <v>185.31</v>
+      </c>
+      <c r="G638" t="n">
+        <v>165.16</v>
+      </c>
+      <c r="H638" t="n">
+        <v>156.85</v>
+      </c>
+      <c r="I638" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J638" t="b">
+        <v>0</v>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 172.74 &lt;= Upper 185.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>305.06</v>
+      </c>
+      <c r="E639" t="n">
+        <v>321.51</v>
+      </c>
+      <c r="F639" t="n">
+        <v>321.51</v>
+      </c>
+      <c r="G639" t="n">
+        <v>312.78</v>
+      </c>
+      <c r="H639" t="n">
+        <v>324.94</v>
+      </c>
+      <c r="I639" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J639" t="b">
+        <v>0</v>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 312.78 &lt;= EMA21 324.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>490</v>
+      </c>
+      <c r="E640" t="n">
+        <v>678.04</v>
+      </c>
+      <c r="F640" t="n">
+        <v>678.04</v>
+      </c>
+      <c r="G640" t="n">
+        <v>532.85</v>
+      </c>
+      <c r="H640" t="n">
+        <v>557.49</v>
+      </c>
+      <c r="I640" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J640" t="b">
+        <v>0</v>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 532.85 &lt;= EMA21 557.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>284.6</v>
+      </c>
+      <c r="E641" t="n">
+        <v>352.3</v>
+      </c>
+      <c r="F641" t="n">
+        <v>352.3</v>
+      </c>
+      <c r="G641" t="n">
+        <v>304.02</v>
+      </c>
+      <c r="H641" t="n">
+        <v>316.71</v>
+      </c>
+      <c r="I641" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J641" t="b">
+        <v>0</v>
+      </c>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 304.02 &lt;= EMA21 316.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>393.22</v>
+      </c>
+      <c r="E642" t="n">
+        <v>449.62</v>
+      </c>
+      <c r="F642" t="n">
+        <v>449.62</v>
+      </c>
+      <c r="G642" t="n">
+        <v>407.21</v>
+      </c>
+      <c r="H642" t="n">
+        <v>410.24</v>
+      </c>
+      <c r="I642" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J642" t="b">
+        <v>0</v>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 407.21 &lt;= EMA21 410.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>206.62</v>
+      </c>
+      <c r="E643" t="n">
+        <v>278.47</v>
+      </c>
+      <c r="F643" t="n">
+        <v>278.47</v>
+      </c>
+      <c r="G643" t="n">
+        <v>230.84</v>
+      </c>
+      <c r="H643" t="n">
+        <v>238.63</v>
+      </c>
+      <c r="I643" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J643" t="b">
+        <v>0</v>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 230.84 &lt;= EMA21 238.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J644" t="b">
+        <v>0</v>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>128.89</v>
+      </c>
+      <c r="E645" t="n">
+        <v>164.54</v>
+      </c>
+      <c r="F645" t="n">
+        <v>164.54</v>
+      </c>
+      <c r="G645" t="n">
+        <v>143.12</v>
+      </c>
+      <c r="H645" t="n">
+        <v>145.4</v>
+      </c>
+      <c r="I645" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J645" t="b">
+        <v>0</v>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 143.12 &lt;= EMA21 145.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>342.68</v>
+      </c>
+      <c r="E646" t="n">
+        <v>390.85</v>
+      </c>
+      <c r="F646" t="n">
+        <v>390.85</v>
+      </c>
+      <c r="G646" t="n">
+        <v>358.92</v>
+      </c>
+      <c r="H646" t="n">
+        <v>350.86</v>
+      </c>
+      <c r="I646" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J646" t="b">
+        <v>0</v>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 342.68 &lt;= Upper 390.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>142.1</v>
+      </c>
+      <c r="E647" t="n">
+        <v>161.39</v>
+      </c>
+      <c r="F647" t="n">
+        <v>161.39</v>
+      </c>
+      <c r="G647" t="n">
+        <v>150.12</v>
+      </c>
+      <c r="H647" t="n">
+        <v>149.19</v>
+      </c>
+      <c r="I647" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J647" t="b">
+        <v>0</v>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 142.10 &lt;= Upper 161.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D648" t="n">
+        <v>169.69</v>
+      </c>
+      <c r="E648" t="n">
+        <v>206.94</v>
+      </c>
+      <c r="F648" t="n">
+        <v>206.94</v>
+      </c>
+      <c r="G648" t="n">
+        <v>184.2</v>
+      </c>
+      <c r="H648" t="n">
+        <v>183.98</v>
+      </c>
+      <c r="I648" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J648" t="b">
+        <v>0</v>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 169.69 &lt;= Upper 206.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D649" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="E649" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="F649" t="n">
+        <v>66.36</v>
+      </c>
+      <c r="G649" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="H649" t="n">
+        <v>60.25</v>
+      </c>
+      <c r="I649" t="n">
+        <v>1</v>
+      </c>
+      <c r="J649" t="b">
+        <v>0</v>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 58.20 &lt;= Upper 66.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D650" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="E650" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="F650" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="G650" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="H650" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="I650" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J650" t="b">
+        <v>0</v>
+      </c>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.61 &lt;= EMA21 11.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>114.68</v>
+      </c>
+      <c r="E651" t="n">
+        <v>123.83</v>
+      </c>
+      <c r="F651" t="n">
+        <v>123.83</v>
+      </c>
+      <c r="G651" t="n">
+        <v>115.05</v>
+      </c>
+      <c r="H651" t="n">
+        <v>110.78</v>
+      </c>
+      <c r="I651" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J651" t="b">
+        <v>0</v>
+      </c>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 114.68 &lt;= Upper 123.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>29.76</v>
+      </c>
+      <c r="E652" t="n">
+        <v>31.87</v>
+      </c>
+      <c r="F652" t="n">
+        <v>31.87</v>
+      </c>
+      <c r="G652" t="n">
+        <v>30.15</v>
+      </c>
+      <c r="H652" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="I652" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J652" t="b">
+        <v>0</v>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 29.76 &lt;= Upper 31.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>142.37</v>
+      </c>
+      <c r="E653" t="n">
+        <v>156.44</v>
+      </c>
+      <c r="F653" t="n">
+        <v>156.44</v>
+      </c>
+      <c r="G653" t="n">
+        <v>146.51</v>
+      </c>
+      <c r="H653" t="n">
+        <v>143.91</v>
+      </c>
+      <c r="I653" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J653" t="b">
+        <v>0</v>
+      </c>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 142.37 &lt;= Upper 156.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>404.63</v>
+      </c>
+      <c r="E654" t="n">
+        <v>419.98</v>
+      </c>
+      <c r="F654" t="n">
+        <v>419.98</v>
+      </c>
+      <c r="G654" t="n">
+        <v>395.51</v>
+      </c>
+      <c r="H654" t="n">
+        <v>396.66</v>
+      </c>
+      <c r="I654" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J654" t="b">
+        <v>0</v>
+      </c>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 395.51 &lt;= EMA21 396.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J655" t="b">
+        <v>0</v>
+      </c>
+      <c r="K655" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>110.75</v>
+      </c>
+      <c r="E656" t="n">
+        <v>125.46</v>
+      </c>
+      <c r="F656" t="n">
+        <v>125.46</v>
+      </c>
+      <c r="G656" t="n">
+        <v>107.87</v>
+      </c>
+      <c r="H656" t="n">
+        <v>110.47</v>
+      </c>
+      <c r="I656" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J656" t="b">
+        <v>0</v>
+      </c>
+      <c r="K656" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.87 &lt;= EMA21 110.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J657" t="b">
+        <v>0</v>
+      </c>
+      <c r="K657" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>211.14</v>
+      </c>
+      <c r="E658" t="n">
+        <v>254.6</v>
+      </c>
+      <c r="F658" t="n">
+        <v>254.6</v>
+      </c>
+      <c r="G658" t="n">
+        <v>218.75</v>
+      </c>
+      <c r="H658" t="n">
+        <v>227.02</v>
+      </c>
+      <c r="I658" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J658" t="b">
+        <v>0</v>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 218.75 &lt;= EMA21 227.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>44.52</v>
+      </c>
+      <c r="E659" t="n">
+        <v>44.54</v>
+      </c>
+      <c r="F659" t="n">
+        <v>44.54</v>
+      </c>
+      <c r="G659" t="n">
+        <v>42.12</v>
+      </c>
+      <c r="H659" t="n">
+        <v>41.18</v>
+      </c>
+      <c r="I659" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J659" t="b">
+        <v>0</v>
+      </c>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 44.52 &lt;= Upper 44.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="E660" t="n">
+        <v>48.45</v>
+      </c>
+      <c r="F660" t="n">
+        <v>48.45</v>
+      </c>
+      <c r="G660" t="n">
+        <v>42.55</v>
+      </c>
+      <c r="H660" t="n">
+        <v>42.11</v>
+      </c>
+      <c r="I660" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J660" t="b">
+        <v>0</v>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 42.54 &lt;= Upper 48.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>76.03</v>
+      </c>
+      <c r="E661" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="F661" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="G661" t="n">
+        <v>79.08</v>
+      </c>
+      <c r="H661" t="n">
+        <v>78.65000000000001</v>
+      </c>
+      <c r="I661" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J661" t="b">
+        <v>0</v>
+      </c>
+      <c r="K661" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 76.03 &lt;= Upper 84.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>104.18</v>
+      </c>
+      <c r="E662" t="n">
+        <v>111.19</v>
+      </c>
+      <c r="F662" t="n">
+        <v>111.19</v>
+      </c>
+      <c r="G662" t="n">
+        <v>106.14</v>
+      </c>
+      <c r="H662" t="n">
+        <v>105.63</v>
+      </c>
+      <c r="I662" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J662" t="b">
+        <v>0</v>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 104.18 &lt;= Upper 111.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>27.91</v>
+      </c>
+      <c r="E663" t="n">
+        <v>29.09</v>
+      </c>
+      <c r="F663" t="n">
+        <v>29.09</v>
+      </c>
+      <c r="G663" t="n">
+        <v>28.26</v>
+      </c>
+      <c r="H663" t="n">
+        <v>28.06</v>
+      </c>
+      <c r="I663" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J663" t="b">
+        <v>0</v>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 27.91 &lt;= Upper 29.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="E664" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="F664" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="G664" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H664" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I664" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J664" t="b">
+        <v>0</v>
+      </c>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1.10 &lt;= EMA21 1.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>523</v>
+      </c>
+      <c r="E665" t="n">
+        <v>572.8</v>
+      </c>
+      <c r="F665" t="n">
+        <v>572.8</v>
+      </c>
+      <c r="G665" t="n">
+        <v>537.99</v>
+      </c>
+      <c r="H665" t="n">
+        <v>530.0700000000001</v>
+      </c>
+      <c r="I665" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J665" t="b">
+        <v>0</v>
+      </c>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 523.00 &lt;= Upper 572.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>7.89</v>
+      </c>
+      <c r="E666" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="F666" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G666" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="H666" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="I666" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J666" t="b">
+        <v>0</v>
+      </c>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8.26 &lt;= EMA21 8.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D667" t="n">
+        <v>105.83</v>
+      </c>
+      <c r="E667" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="F667" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="G667" t="n">
+        <v>106.32</v>
+      </c>
+      <c r="H667" t="n">
+        <v>107.63</v>
+      </c>
+      <c r="I667" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J667" t="b">
+        <v>0</v>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.32 &lt;= EMA21 107.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D668" t="n">
+        <v>902.6</v>
+      </c>
+      <c r="E668" t="n">
+        <v>980.83</v>
+      </c>
+      <c r="F668" t="n">
+        <v>980.83</v>
+      </c>
+      <c r="G668" t="n">
+        <v>924.5700000000001</v>
+      </c>
+      <c r="H668" t="n">
+        <v>936.24</v>
+      </c>
+      <c r="I668" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J668" t="b">
+        <v>0</v>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 924.57 &lt;= EMA21 936.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D669" t="n">
+        <v>157.52</v>
+      </c>
+      <c r="E669" t="n">
+        <v>170.88</v>
+      </c>
+      <c r="F669" t="n">
+        <v>170.88</v>
+      </c>
+      <c r="G669" t="n">
+        <v>161.91</v>
+      </c>
+      <c r="H669" t="n">
+        <v>159</v>
+      </c>
+      <c r="I669" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J669" t="b">
+        <v>0</v>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 157.52 &lt;= Upper 170.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D670" t="n">
+        <v>310.45</v>
+      </c>
+      <c r="E670" t="n">
+        <v>347.76</v>
+      </c>
+      <c r="F670" t="n">
+        <v>347.76</v>
+      </c>
+      <c r="G670" t="n">
+        <v>319.47</v>
+      </c>
+      <c r="H670" t="n">
+        <v>326.44</v>
+      </c>
+      <c r="I670" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J670" t="b">
+        <v>0</v>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 319.47 &lt;= EMA21 326.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D671" t="n">
+        <v>198.6</v>
+      </c>
+      <c r="E671" t="n">
+        <v>225.14</v>
+      </c>
+      <c r="F671" t="n">
+        <v>225.14</v>
+      </c>
+      <c r="G671" t="n">
+        <v>203.48</v>
+      </c>
+      <c r="H671" t="n">
+        <v>207.91</v>
+      </c>
+      <c r="I671" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J671" t="b">
+        <v>0</v>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 203.48 &lt;= EMA21 207.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D672" t="n">
+        <v>56.44</v>
+      </c>
+      <c r="E672" t="n">
+        <v>59.38</v>
+      </c>
+      <c r="F672" t="n">
+        <v>59.38</v>
+      </c>
+      <c r="G672" t="n">
+        <v>57.58</v>
+      </c>
+      <c r="H672" t="n">
+        <v>57.53</v>
+      </c>
+      <c r="I672" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J672" t="b">
+        <v>0</v>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 56.44 &lt;= Upper 59.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D673" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="E673" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="F673" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="G673" t="n">
+        <v>12.28</v>
+      </c>
+      <c r="H673" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="I673" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J673" t="b">
+        <v>0</v>
+      </c>
+      <c r="K673" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12.28 &lt;= EMA21 12.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D674" t="n">
+        <v>124.57</v>
+      </c>
+      <c r="E674" t="n">
+        <v>133.03</v>
+      </c>
+      <c r="F674" t="n">
+        <v>133.03</v>
+      </c>
+      <c r="G674" t="n">
+        <v>127.68</v>
+      </c>
+      <c r="H674" t="n">
+        <v>126</v>
+      </c>
+      <c r="I674" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J674" t="b">
+        <v>0</v>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 124.57 &lt;= Upper 133.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D675" t="n">
+        <v>118.39</v>
+      </c>
+      <c r="E675" t="n">
+        <v>137.37</v>
+      </c>
+      <c r="F675" t="n">
+        <v>137.37</v>
+      </c>
+      <c r="G675" t="n">
+        <v>127.2</v>
+      </c>
+      <c r="H675" t="n">
+        <v>128.42</v>
+      </c>
+      <c r="I675" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="J675" t="b">
+        <v>0</v>
+      </c>
+      <c r="K675" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 127.20 &lt;= EMA21 128.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>88.51000000000001</v>
+      </c>
+      <c r="E676" t="n">
+        <v>97.22</v>
+      </c>
+      <c r="F676" t="n">
+        <v>97.22</v>
+      </c>
+      <c r="G676" t="n">
+        <v>91.41</v>
+      </c>
+      <c r="H676" t="n">
+        <v>92.45999999999999</v>
+      </c>
+      <c r="I676" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J676" t="b">
+        <v>0</v>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 91.41 &lt;= EMA21 92.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>225.27</v>
+      </c>
+      <c r="E677" t="n">
+        <v>247.52</v>
+      </c>
+      <c r="F677" t="n">
+        <v>247.52</v>
+      </c>
+      <c r="G677" t="n">
+        <v>230.05</v>
+      </c>
+      <c r="H677" t="n">
+        <v>233.75</v>
+      </c>
+      <c r="I677" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J677" t="b">
+        <v>0</v>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 230.05 &lt;= EMA21 233.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>126.12</v>
+      </c>
+      <c r="E678" t="n">
+        <v>156.65</v>
+      </c>
+      <c r="F678" t="n">
+        <v>156.65</v>
+      </c>
+      <c r="G678" t="n">
+        <v>132.22</v>
+      </c>
+      <c r="H678" t="n">
+        <v>138.63</v>
+      </c>
+      <c r="I678" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J678" t="b">
+        <v>0</v>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 132.22 &lt;= EMA21 138.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D679" t="n">
+        <v>37.35</v>
+      </c>
+      <c r="E679" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="F679" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="G679" t="n">
+        <v>38.35</v>
+      </c>
+      <c r="H679" t="n">
+        <v>39.19</v>
+      </c>
+      <c r="I679" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J679" t="b">
+        <v>0</v>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 38.35 &lt;= EMA21 39.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D680" t="n">
+        <v>99.72</v>
+      </c>
+      <c r="E680" t="n">
+        <v>130.21</v>
+      </c>
+      <c r="F680" t="n">
+        <v>130.21</v>
+      </c>
+      <c r="G680" t="n">
+        <v>110.6</v>
+      </c>
+      <c r="H680" t="n">
+        <v>115.04</v>
+      </c>
+      <c r="I680" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J680" t="b">
+        <v>0</v>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 110.60 &lt;= EMA21 115.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D681" t="n">
+        <v>100.04</v>
+      </c>
+      <c r="E681" t="n">
+        <v>110.39</v>
+      </c>
+      <c r="F681" t="n">
+        <v>110.39</v>
+      </c>
+      <c r="G681" t="n">
+        <v>104.24</v>
+      </c>
+      <c r="H681" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="I681" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J681" t="b">
+        <v>0</v>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 104.24 &lt;= EMA21 105.15)</t>
         </is>
       </c>
     </row>
@@ -25172,7 +29418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25486,6 +29732,68 @@
         <v>1.52</v>
       </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>653.6900000000001</v>
+      </c>
+      <c r="E11" t="n">
+        <v>624.27</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>168.46</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -25565,34 +29873,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>524.14</v>
+        <v>174.09</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>1572.42</v>
+        <v>1914.99</v>
       </c>
       <c r="F2" t="n">
-        <v>524.14</v>
+        <v>174.09</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>500.55</v>
+        <v>166.26</v>
       </c>
       <c r="I2" t="n">
-        <v>524.14</v>
+        <v>174.09</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -25606,7 +29914,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -25615,25 +29923,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>174.09</v>
+        <v>162.52</v>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>1914.99</v>
+        <v>1950.24</v>
       </c>
       <c r="F3" t="n">
-        <v>174.09</v>
+        <v>162.52</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>166.26</v>
+        <v>155.21</v>
       </c>
       <c r="I3" t="n">
-        <v>174.09</v>
+        <v>162.52</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -25647,7 +29955,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>QRVO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -25656,25 +29964,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>162.52</v>
+        <v>104.07</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
-        <v>1950.24</v>
+        <v>1977.33</v>
       </c>
       <c r="F4" t="n">
-        <v>162.52</v>
+        <v>104.07</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>155.21</v>
+        <v>99.39</v>
       </c>
       <c r="I4" t="n">
-        <v>162.52</v>
+        <v>104.07</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -25688,34 +29996,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>QRVO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>104.07</v>
+        <v>653.6900000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>1977.33</v>
+        <v>1961.07</v>
       </c>
       <c r="F5" t="n">
-        <v>104.07</v>
+        <v>653.6900000000001</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>99.39</v>
+        <v>624.27</v>
       </c>
       <c r="I5" t="n">
-        <v>104.07</v>
+        <v>653.6900000000001</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -25737,7 +30045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25904,6 +30212,57 @@
         <v>2</v>
       </c>
       <c r="M3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>524.14</v>
+      </c>
+      <c r="E4" t="n">
+        <v>537.66</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1572.42</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2.579</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2.529</v>
+      </c>
+      <c r="J4" t="n">
+        <v>39.77</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>TRAILING_STOP</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -25920,7 +30279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26318,6 +30677,104 @@
         </is>
       </c>
       <c r="K8" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:43:35</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>27F84F6838</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>537.66</v>
+      </c>
+      <c r="G9" t="n">
+        <v>537.66</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>TRAILING_STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:43:35</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>193A12ACFF</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>653.6900000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>653.6900000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
         </is>
@@ -26402,7 +30859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26782,6 +31239,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>04:43:36</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2064.86</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7803.63</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9868.49</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-131.51</v>
+      </c>
+      <c r="G12" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-12T04:45 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K781"/>
+  <dimension ref="A1:K881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33650,6 +33650,4234 @@
       <c r="K781" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 103.24 &lt;= EMA21 104.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="J782" t="b">
+        <v>0</v>
+      </c>
+      <c r="K782" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D783" t="n">
+        <v>495.63</v>
+      </c>
+      <c r="E783" t="n">
+        <v>514.13</v>
+      </c>
+      <c r="F783" t="n">
+        <v>514.13</v>
+      </c>
+      <c r="G783" t="n">
+        <v>496.43</v>
+      </c>
+      <c r="H783" t="n">
+        <v>490.21</v>
+      </c>
+      <c r="I783" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J783" t="b">
+        <v>0</v>
+      </c>
+      <c r="K783" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 495.63 &lt;= Upper 514.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D784" t="n">
+        <v>218.29</v>
+      </c>
+      <c r="E784" t="n">
+        <v>232.14</v>
+      </c>
+      <c r="F784" t="n">
+        <v>232.14</v>
+      </c>
+      <c r="G784" t="n">
+        <v>221.48</v>
+      </c>
+      <c r="H784" t="n">
+        <v>219.52</v>
+      </c>
+      <c r="I784" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J784" t="b">
+        <v>0</v>
+      </c>
+      <c r="K784" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 218.29 &lt;= Upper 232.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D785" t="n">
+        <v>338.5</v>
+      </c>
+      <c r="E785" t="n">
+        <v>350.41</v>
+      </c>
+      <c r="F785" t="n">
+        <v>350.41</v>
+      </c>
+      <c r="G785" t="n">
+        <v>337.39</v>
+      </c>
+      <c r="H785" t="n">
+        <v>340.75</v>
+      </c>
+      <c r="I785" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J785" t="b">
+        <v>0</v>
+      </c>
+      <c r="K785" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 337.39 &lt;= EMA21 340.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="D786" t="n">
+        <v>335.45</v>
+      </c>
+      <c r="E786" t="n">
+        <v>347.04</v>
+      </c>
+      <c r="F786" t="n">
+        <v>347.04</v>
+      </c>
+      <c r="G786" t="n">
+        <v>334.51</v>
+      </c>
+      <c r="H786" t="n">
+        <v>338.01</v>
+      </c>
+      <c r="I786" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J786" t="b">
+        <v>0</v>
+      </c>
+      <c r="K786" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 334.51 &lt;= EMA21 338.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D787" t="n">
+        <v>256.78</v>
+      </c>
+      <c r="E787" t="n">
+        <v>266.66</v>
+      </c>
+      <c r="F787" t="n">
+        <v>266.66</v>
+      </c>
+      <c r="G787" t="n">
+        <v>256.35</v>
+      </c>
+      <c r="H787" t="n">
+        <v>257.94</v>
+      </c>
+      <c r="I787" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J787" t="b">
+        <v>0</v>
+      </c>
+      <c r="K787" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 256.35 &lt;= EMA21 257.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D788" t="n">
+        <v>648.03</v>
+      </c>
+      <c r="E788" t="n">
+        <v>655.15</v>
+      </c>
+      <c r="F788" t="n">
+        <v>655.15</v>
+      </c>
+      <c r="G788" t="n">
+        <v>620.72</v>
+      </c>
+      <c r="H788" t="n">
+        <v>601.79</v>
+      </c>
+      <c r="I788" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J788" t="b">
+        <v>0</v>
+      </c>
+      <c r="K788" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 648.03 &lt;= Upper 655.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D789" t="n">
+        <v>365.44</v>
+      </c>
+      <c r="E789" t="n">
+        <v>376.86</v>
+      </c>
+      <c r="F789" t="n">
+        <v>376.86</v>
+      </c>
+      <c r="G789" t="n">
+        <v>362.41</v>
+      </c>
+      <c r="H789" t="n">
+        <v>356.24</v>
+      </c>
+      <c r="I789" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J789" t="b">
+        <v>0</v>
+      </c>
+      <c r="K789" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 365.44 &lt;= Upper 376.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D790" t="n">
+        <v>361.99</v>
+      </c>
+      <c r="E790" t="n">
+        <v>388.6</v>
+      </c>
+      <c r="F790" t="n">
+        <v>388.6</v>
+      </c>
+      <c r="G790" t="n">
+        <v>364.13</v>
+      </c>
+      <c r="H790" t="n">
+        <v>370.81</v>
+      </c>
+      <c r="I790" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J790" t="b">
+        <v>0</v>
+      </c>
+      <c r="K790" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 364.13 &lt;= EMA21 370.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D791" t="n">
+        <v>150.28</v>
+      </c>
+      <c r="E791" t="n">
+        <v>161.93</v>
+      </c>
+      <c r="F791" t="n">
+        <v>161.93</v>
+      </c>
+      <c r="G791" t="n">
+        <v>153.35</v>
+      </c>
+      <c r="H791" t="n">
+        <v>150.03</v>
+      </c>
+      <c r="I791" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="J791" t="b">
+        <v>0</v>
+      </c>
+      <c r="K791" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 150.28 &lt;= Upper 161.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D792" t="n">
+        <v>247.72</v>
+      </c>
+      <c r="E792" t="n">
+        <v>284.07</v>
+      </c>
+      <c r="F792" t="n">
+        <v>284.07</v>
+      </c>
+      <c r="G792" t="n">
+        <v>246.44</v>
+      </c>
+      <c r="H792" t="n">
+        <v>232.44</v>
+      </c>
+      <c r="I792" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J792" t="b">
+        <v>0</v>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 247.72 &lt;= Upper 284.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D793" t="n">
+        <v>252.23</v>
+      </c>
+      <c r="E793" t="n">
+        <v>298.7</v>
+      </c>
+      <c r="F793" t="n">
+        <v>298.7</v>
+      </c>
+      <c r="G793" t="n">
+        <v>263.56</v>
+      </c>
+      <c r="H793" t="n">
+        <v>266.24</v>
+      </c>
+      <c r="I793" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="J793" t="b">
+        <v>0</v>
+      </c>
+      <c r="K793" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 263.56 &lt;= EMA21 266.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>516.13</v>
+      </c>
+      <c r="E794" t="n">
+        <v>524.87</v>
+      </c>
+      <c r="F794" t="n">
+        <v>524.87</v>
+      </c>
+      <c r="G794" t="n">
+        <v>494.1</v>
+      </c>
+      <c r="H794" t="n">
+        <v>487.01</v>
+      </c>
+      <c r="I794" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J794" t="b">
+        <v>0</v>
+      </c>
+      <c r="K794" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 516.13 &lt;= Upper 524.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>102.94</v>
+      </c>
+      <c r="E795" t="n">
+        <v>107.4</v>
+      </c>
+      <c r="F795" t="n">
+        <v>107.4</v>
+      </c>
+      <c r="G795" t="n">
+        <v>98.52</v>
+      </c>
+      <c r="H795" t="n">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="I795" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J795" t="b">
+        <v>0</v>
+      </c>
+      <c r="K795" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 102.94 &lt;= Upper 107.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D796" t="n">
+        <v>975.26</v>
+      </c>
+      <c r="E796" t="n">
+        <v>1026.84</v>
+      </c>
+      <c r="F796" t="n">
+        <v>1026.84</v>
+      </c>
+      <c r="G796" t="n">
+        <v>978.64</v>
+      </c>
+      <c r="H796" t="n">
+        <v>959.4400000000001</v>
+      </c>
+      <c r="I796" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J796" t="b">
+        <v>0</v>
+      </c>
+      <c r="K796" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 975.26 &lt;= Upper 1026.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D797" t="n">
+        <v>181.97</v>
+      </c>
+      <c r="E797" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="F797" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="G797" t="n">
+        <v>173.18</v>
+      </c>
+      <c r="H797" t="n">
+        <v>168.95</v>
+      </c>
+      <c r="I797" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J797" t="b">
+        <v>0</v>
+      </c>
+      <c r="K797" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.05x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="D798" t="n">
+        <v>268.7</v>
+      </c>
+      <c r="E798" t="n">
+        <v>279.13</v>
+      </c>
+      <c r="F798" t="n">
+        <v>279.13</v>
+      </c>
+      <c r="G798" t="n">
+        <v>261.24</v>
+      </c>
+      <c r="H798" t="n">
+        <v>264.45</v>
+      </c>
+      <c r="I798" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J798" t="b">
+        <v>0</v>
+      </c>
+      <c r="K798" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 261.24 &lt;= EMA21 264.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D799" t="n">
+        <v>456.49</v>
+      </c>
+      <c r="E799" t="n">
+        <v>527.9299999999999</v>
+      </c>
+      <c r="F799" t="n">
+        <v>527.9299999999999</v>
+      </c>
+      <c r="G799" t="n">
+        <v>460.43</v>
+      </c>
+      <c r="H799" t="n">
+        <v>475.94</v>
+      </c>
+      <c r="I799" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J799" t="b">
+        <v>0</v>
+      </c>
+      <c r="K799" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 460.43 &lt;= EMA21 475.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D800" t="n">
+        <v>298.22</v>
+      </c>
+      <c r="E800" t="n">
+        <v>338.71</v>
+      </c>
+      <c r="F800" t="n">
+        <v>338.71</v>
+      </c>
+      <c r="G800" t="n">
+        <v>304.39</v>
+      </c>
+      <c r="H800" t="n">
+        <v>307.79</v>
+      </c>
+      <c r="I800" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J800" t="b">
+        <v>0</v>
+      </c>
+      <c r="K800" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 304.39 &lt;= EMA21 307.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D801" t="n">
+        <v>180.64</v>
+      </c>
+      <c r="E801" t="n">
+        <v>202.46</v>
+      </c>
+      <c r="F801" t="n">
+        <v>202.46</v>
+      </c>
+      <c r="G801" t="n">
+        <v>180.69</v>
+      </c>
+      <c r="H801" t="n">
+        <v>184.64</v>
+      </c>
+      <c r="I801" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J801" t="b">
+        <v>0</v>
+      </c>
+      <c r="K801" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 180.69 &lt;= EMA21 184.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D802" t="n">
+        <v>1698.3</v>
+      </c>
+      <c r="E802" t="n">
+        <v>1852.66</v>
+      </c>
+      <c r="F802" t="n">
+        <v>1852.66</v>
+      </c>
+      <c r="G802" t="n">
+        <v>1709.16</v>
+      </c>
+      <c r="H802" t="n">
+        <v>1722.07</v>
+      </c>
+      <c r="I802" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J802" t="b">
+        <v>0</v>
+      </c>
+      <c r="K802" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1709.16 &lt;= EMA21 1722.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D803" t="n">
+        <v>378.78</v>
+      </c>
+      <c r="E803" t="n">
+        <v>388</v>
+      </c>
+      <c r="F803" t="n">
+        <v>388</v>
+      </c>
+      <c r="G803" t="n">
+        <v>365.96</v>
+      </c>
+      <c r="H803" t="n">
+        <v>368.14</v>
+      </c>
+      <c r="I803" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J803" t="b">
+        <v>0</v>
+      </c>
+      <c r="K803" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.96 &lt;= EMA21 368.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D804" t="n">
+        <v>236.1</v>
+      </c>
+      <c r="E804" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="F804" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="G804" t="n">
+        <v>226.57</v>
+      </c>
+      <c r="H804" t="n">
+        <v>224.15</v>
+      </c>
+      <c r="I804" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J804" t="b">
+        <v>0</v>
+      </c>
+      <c r="K804" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 236.10 &lt;= Upper 253.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="D805" t="n">
+        <v>236.62</v>
+      </c>
+      <c r="E805" t="n">
+        <v>234.54</v>
+      </c>
+      <c r="F805" t="n">
+        <v>234.54</v>
+      </c>
+      <c r="G805" t="n">
+        <v>227.64</v>
+      </c>
+      <c r="H805" t="n">
+        <v>229.77</v>
+      </c>
+      <c r="I805" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J805" t="b">
+        <v>0</v>
+      </c>
+      <c r="K805" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 227.64 &lt;= EMA21 229.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D806" t="n">
+        <v>76.14</v>
+      </c>
+      <c r="E806" t="n">
+        <v>81.75</v>
+      </c>
+      <c r="F806" t="n">
+        <v>81.75</v>
+      </c>
+      <c r="G806" t="n">
+        <v>73.11</v>
+      </c>
+      <c r="H806" t="n">
+        <v>75.22</v>
+      </c>
+      <c r="I806" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="J806" t="b">
+        <v>0</v>
+      </c>
+      <c r="K806" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 73.11 &lt;= EMA21 75.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
+      <c r="D807" t="n">
+        <v>1234.46</v>
+      </c>
+      <c r="E807" t="n">
+        <v>1403.2</v>
+      </c>
+      <c r="F807" t="n">
+        <v>1403.2</v>
+      </c>
+      <c r="G807" t="n">
+        <v>1228.68</v>
+      </c>
+      <c r="H807" t="n">
+        <v>1266.58</v>
+      </c>
+      <c r="I807" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J807" t="b">
+        <v>0</v>
+      </c>
+      <c r="K807" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1228.68 &lt;= EMA21 1266.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D808" t="n">
+        <v>88.34999999999999</v>
+      </c>
+      <c r="E808" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="F808" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="G808" t="n">
+        <v>77.19</v>
+      </c>
+      <c r="H808" t="n">
+        <v>72.43000000000001</v>
+      </c>
+      <c r="I808" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="J808" t="b">
+        <v>1</v>
+      </c>
+      <c r="K808" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D809" t="n">
+        <v>116.65</v>
+      </c>
+      <c r="E809" t="n">
+        <v>111.63</v>
+      </c>
+      <c r="F809" t="n">
+        <v>111.63</v>
+      </c>
+      <c r="G809" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="H809" t="n">
+        <v>100.92</v>
+      </c>
+      <c r="I809" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="J809" t="b">
+        <v>1</v>
+      </c>
+      <c r="K809" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="D810" t="n">
+        <v>379.72</v>
+      </c>
+      <c r="E810" t="n">
+        <v>425.35</v>
+      </c>
+      <c r="F810" t="n">
+        <v>425.35</v>
+      </c>
+      <c r="G810" t="n">
+        <v>367.51</v>
+      </c>
+      <c r="H810" t="n">
+        <v>368.52</v>
+      </c>
+      <c r="I810" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J810" t="b">
+        <v>0</v>
+      </c>
+      <c r="K810" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 367.51 &lt;= EMA21 368.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>ENTG</t>
+        </is>
+      </c>
+      <c r="D811" t="n">
+        <v>140.37</v>
+      </c>
+      <c r="E811" t="n">
+        <v>159.41</v>
+      </c>
+      <c r="F811" t="n">
+        <v>159.41</v>
+      </c>
+      <c r="G811" t="n">
+        <v>138.76</v>
+      </c>
+      <c r="H811" t="n">
+        <v>139.93</v>
+      </c>
+      <c r="I811" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J811" t="b">
+        <v>0</v>
+      </c>
+      <c r="K811" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 138.76 &lt;= EMA21 139.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>MCHP</t>
+        </is>
+      </c>
+      <c r="D812" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="E812" t="n">
+        <v>79.02</v>
+      </c>
+      <c r="F812" t="n">
+        <v>79.02</v>
+      </c>
+      <c r="G812" t="n">
+        <v>73.37</v>
+      </c>
+      <c r="H812" t="n">
+        <v>74.66</v>
+      </c>
+      <c r="I812" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J812" t="b">
+        <v>0</v>
+      </c>
+      <c r="K812" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 73.37 &lt;= EMA21 74.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D813" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="E813" t="n">
+        <v>40.57</v>
+      </c>
+      <c r="F813" t="n">
+        <v>40.57</v>
+      </c>
+      <c r="G813" t="n">
+        <v>38.54</v>
+      </c>
+      <c r="H813" t="n">
+        <v>37.13</v>
+      </c>
+      <c r="I813" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J813" t="b">
+        <v>0</v>
+      </c>
+      <c r="K813" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 40.10 &lt;= Upper 40.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D814" t="n">
+        <v>567.29</v>
+      </c>
+      <c r="E814" t="n">
+        <v>559.79</v>
+      </c>
+      <c r="F814" t="n">
+        <v>559.79</v>
+      </c>
+      <c r="G814" t="n">
+        <v>514.6900000000001</v>
+      </c>
+      <c r="H814" t="n">
+        <v>487.27</v>
+      </c>
+      <c r="I814" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J814" t="b">
+        <v>1</v>
+      </c>
+      <c r="K814" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D815" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="E815" t="n">
+        <v>34</v>
+      </c>
+      <c r="F815" t="n">
+        <v>34</v>
+      </c>
+      <c r="G815" t="n">
+        <v>32.28</v>
+      </c>
+      <c r="H815" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="I815" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="J815" t="b">
+        <v>1</v>
+      </c>
+      <c r="K815" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="D816" t="n">
+        <v>447.18</v>
+      </c>
+      <c r="E816" t="n">
+        <v>514.9</v>
+      </c>
+      <c r="F816" t="n">
+        <v>514.9</v>
+      </c>
+      <c r="G816" t="n">
+        <v>460.84</v>
+      </c>
+      <c r="H816" t="n">
+        <v>467.52</v>
+      </c>
+      <c r="I816" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J816" t="b">
+        <v>0</v>
+      </c>
+      <c r="K816" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 460.84 &lt;= EMA21 467.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D817" t="n">
+        <v>830.17</v>
+      </c>
+      <c r="E817" t="n">
+        <v>962.65</v>
+      </c>
+      <c r="F817" t="n">
+        <v>962.65</v>
+      </c>
+      <c r="G817" t="n">
+        <v>849.84</v>
+      </c>
+      <c r="H817" t="n">
+        <v>849.6</v>
+      </c>
+      <c r="I817" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J817" t="b">
+        <v>0</v>
+      </c>
+      <c r="K817" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 830.17 &lt;= Upper 962.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="D818" t="n">
+        <v>199.59</v>
+      </c>
+      <c r="E818" t="n">
+        <v>204.19</v>
+      </c>
+      <c r="F818" t="n">
+        <v>204.19</v>
+      </c>
+      <c r="G818" t="n">
+        <v>193.65</v>
+      </c>
+      <c r="H818" t="n">
+        <v>192.18</v>
+      </c>
+      <c r="I818" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J818" t="b">
+        <v>0</v>
+      </c>
+      <c r="K818" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 199.59 &lt;= Upper 204.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D819" t="n">
+        <v>112.13</v>
+      </c>
+      <c r="E819" t="n">
+        <v>113.28</v>
+      </c>
+      <c r="F819" t="n">
+        <v>113.28</v>
+      </c>
+      <c r="G819" t="n">
+        <v>109.92</v>
+      </c>
+      <c r="H819" t="n">
+        <v>111.19</v>
+      </c>
+      <c r="I819" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J819" t="b">
+        <v>0</v>
+      </c>
+      <c r="K819" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 109.92 &lt;= EMA21 111.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="D820" t="n">
+        <v>183.9</v>
+      </c>
+      <c r="E820" t="n">
+        <v>195.42</v>
+      </c>
+      <c r="F820" t="n">
+        <v>195.42</v>
+      </c>
+      <c r="G820" t="n">
+        <v>182.83</v>
+      </c>
+      <c r="H820" t="n">
+        <v>180.81</v>
+      </c>
+      <c r="I820" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J820" t="b">
+        <v>0</v>
+      </c>
+      <c r="K820" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 183.90 &lt;= Upper 195.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="D821" t="n">
+        <v>243.29</v>
+      </c>
+      <c r="E821" t="n">
+        <v>241.32</v>
+      </c>
+      <c r="F821" t="n">
+        <v>241.32</v>
+      </c>
+      <c r="G821" t="n">
+        <v>236.36</v>
+      </c>
+      <c r="H821" t="n">
+        <v>235.04</v>
+      </c>
+      <c r="I821" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J821" t="b">
+        <v>0</v>
+      </c>
+      <c r="K821" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.02x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D822" t="n">
+        <v>132.53</v>
+      </c>
+      <c r="E822" t="n">
+        <v>149.94</v>
+      </c>
+      <c r="F822" t="n">
+        <v>149.94</v>
+      </c>
+      <c r="G822" t="n">
+        <v>134.92</v>
+      </c>
+      <c r="H822" t="n">
+        <v>131.87</v>
+      </c>
+      <c r="I822" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J822" t="b">
+        <v>0</v>
+      </c>
+      <c r="K822" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 132.53 &lt;= Upper 149.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>INTU</t>
+        </is>
+      </c>
+      <c r="D823" t="n">
+        <v>321.57</v>
+      </c>
+      <c r="E823" t="n">
+        <v>379.45</v>
+      </c>
+      <c r="F823" t="n">
+        <v>379.45</v>
+      </c>
+      <c r="G823" t="n">
+        <v>328.97</v>
+      </c>
+      <c r="H823" t="n">
+        <v>334.63</v>
+      </c>
+      <c r="I823" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J823" t="b">
+        <v>0</v>
+      </c>
+      <c r="K823" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 328.97 &lt;= EMA21 334.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="D824" t="n">
+        <v>330.65</v>
+      </c>
+      <c r="E824" t="n">
+        <v>392.39</v>
+      </c>
+      <c r="F824" t="n">
+        <v>392.39</v>
+      </c>
+      <c r="G824" t="n">
+        <v>340.61</v>
+      </c>
+      <c r="H824" t="n">
+        <v>347.9</v>
+      </c>
+      <c r="I824" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J824" t="b">
+        <v>0</v>
+      </c>
+      <c r="K824" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 340.61 &lt;= EMA21 347.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D825" t="n">
+        <v>206.74</v>
+      </c>
+      <c r="E825" t="n">
+        <v>233.05</v>
+      </c>
+      <c r="F825" t="n">
+        <v>233.05</v>
+      </c>
+      <c r="G825" t="n">
+        <v>209.5</v>
+      </c>
+      <c r="H825" t="n">
+        <v>208.16</v>
+      </c>
+      <c r="I825" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J825" t="b">
+        <v>0</v>
+      </c>
+      <c r="K825" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 206.74 &lt;= Upper 233.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D826" t="n">
+        <v>328.99</v>
+      </c>
+      <c r="E826" t="n">
+        <v>347.77</v>
+      </c>
+      <c r="F826" t="n">
+        <v>347.77</v>
+      </c>
+      <c r="G826" t="n">
+        <v>330.44</v>
+      </c>
+      <c r="H826" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="I826" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J826" t="b">
+        <v>0</v>
+      </c>
+      <c r="K826" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 328.99 &lt;= Upper 347.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D827" t="n">
+        <v>167.23</v>
+      </c>
+      <c r="E827" t="n">
+        <v>187.99</v>
+      </c>
+      <c r="F827" t="n">
+        <v>187.99</v>
+      </c>
+      <c r="G827" t="n">
+        <v>171.98</v>
+      </c>
+      <c r="H827" t="n">
+        <v>170.73</v>
+      </c>
+      <c r="I827" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J827" t="b">
+        <v>0</v>
+      </c>
+      <c r="K827" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 167.23 &lt;= Upper 187.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>DDOG</t>
+        </is>
+      </c>
+      <c r="D828" t="n">
+        <v>221.21</v>
+      </c>
+      <c r="E828" t="n">
+        <v>254.82</v>
+      </c>
+      <c r="F828" t="n">
+        <v>254.82</v>
+      </c>
+      <c r="G828" t="n">
+        <v>221.61</v>
+      </c>
+      <c r="H828" t="n">
+        <v>229.02</v>
+      </c>
+      <c r="I828" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J828" t="b">
+        <v>0</v>
+      </c>
+      <c r="K828" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 221.61 &lt;= EMA21 229.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>164.54</v>
+      </c>
+      <c r="E829" t="n">
+        <v>193.46</v>
+      </c>
+      <c r="F829" t="n">
+        <v>193.46</v>
+      </c>
+      <c r="G829" t="n">
+        <v>169.35</v>
+      </c>
+      <c r="H829" t="n">
+        <v>171.24</v>
+      </c>
+      <c r="I829" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J829" t="b">
+        <v>0</v>
+      </c>
+      <c r="K829" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 169.35 &lt;= EMA21 171.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D830" t="n">
+        <v>306.53</v>
+      </c>
+      <c r="E830" t="n">
+        <v>321.72</v>
+      </c>
+      <c r="F830" t="n">
+        <v>321.72</v>
+      </c>
+      <c r="G830" t="n">
+        <v>297.95</v>
+      </c>
+      <c r="H830" t="n">
+        <v>294</v>
+      </c>
+      <c r="I830" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J830" t="b">
+        <v>0</v>
+      </c>
+      <c r="K830" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 306.53 &lt;= Upper 321.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="D831" t="n">
+        <v>362.21</v>
+      </c>
+      <c r="E831" t="n">
+        <v>479.22</v>
+      </c>
+      <c r="F831" t="n">
+        <v>479.22</v>
+      </c>
+      <c r="G831" t="n">
+        <v>380.35</v>
+      </c>
+      <c r="H831" t="n">
+        <v>392.25</v>
+      </c>
+      <c r="I831" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J831" t="b">
+        <v>0</v>
+      </c>
+      <c r="K831" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 380.35 &lt;= EMA21 392.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>FTNT</t>
+        </is>
+      </c>
+      <c r="D832" t="n">
+        <v>156.07</v>
+      </c>
+      <c r="E832" t="n">
+        <v>169.82</v>
+      </c>
+      <c r="F832" t="n">
+        <v>169.82</v>
+      </c>
+      <c r="G832" t="n">
+        <v>158.09</v>
+      </c>
+      <c r="H832" t="n">
+        <v>158.56</v>
+      </c>
+      <c r="I832" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J832" t="b">
+        <v>0</v>
+      </c>
+      <c r="K832" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 158.09 &lt;= EMA21 158.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D833" t="n">
+        <v>179.7</v>
+      </c>
+      <c r="E833" t="n">
+        <v>199.3</v>
+      </c>
+      <c r="F833" t="n">
+        <v>199.3</v>
+      </c>
+      <c r="G833" t="n">
+        <v>181.18</v>
+      </c>
+      <c r="H833" t="n">
+        <v>171.55</v>
+      </c>
+      <c r="I833" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J833" t="b">
+        <v>0</v>
+      </c>
+      <c r="K833" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 179.70 &lt;= Upper 199.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>WDAY</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>185.7</v>
+      </c>
+      <c r="E834" t="n">
+        <v>207.69</v>
+      </c>
+      <c r="F834" t="n">
+        <v>207.69</v>
+      </c>
+      <c r="G834" t="n">
+        <v>190.97</v>
+      </c>
+      <c r="H834" t="n">
+        <v>189.38</v>
+      </c>
+      <c r="I834" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J834" t="b">
+        <v>0</v>
+      </c>
+      <c r="K834" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 185.70 &lt;= Upper 207.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>225.33</v>
+      </c>
+      <c r="E835" t="n">
+        <v>266.28</v>
+      </c>
+      <c r="F835" t="n">
+        <v>266.28</v>
+      </c>
+      <c r="G835" t="n">
+        <v>236.8</v>
+      </c>
+      <c r="H835" t="n">
+        <v>237.38</v>
+      </c>
+      <c r="I835" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J835" t="b">
+        <v>0</v>
+      </c>
+      <c r="K835" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 236.80 &lt;= EMA21 237.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>VEEV</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>262.4</v>
+      </c>
+      <c r="E836" t="n">
+        <v>293.57</v>
+      </c>
+      <c r="F836" t="n">
+        <v>293.57</v>
+      </c>
+      <c r="G836" t="n">
+        <v>266.41</v>
+      </c>
+      <c r="H836" t="n">
+        <v>257.91</v>
+      </c>
+      <c r="I836" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J836" t="b">
+        <v>0</v>
+      </c>
+      <c r="K836" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 262.40 &lt;= Upper 293.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>ZM</t>
+        </is>
+      </c>
+      <c r="D837" t="n">
+        <v>95.56999999999999</v>
+      </c>
+      <c r="E837" t="n">
+        <v>109.82</v>
+      </c>
+      <c r="F837" t="n">
+        <v>109.82</v>
+      </c>
+      <c r="G837" t="n">
+        <v>97.15000000000001</v>
+      </c>
+      <c r="H837" t="n">
+        <v>98.52</v>
+      </c>
+      <c r="I837" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J837" t="b">
+        <v>0</v>
+      </c>
+      <c r="K837" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 97.15 &lt;= EMA21 98.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>OKTA</t>
+        </is>
+      </c>
+      <c r="D838" t="n">
+        <v>166.5</v>
+      </c>
+      <c r="E838" t="n">
+        <v>188.33</v>
+      </c>
+      <c r="F838" t="n">
+        <v>188.33</v>
+      </c>
+      <c r="G838" t="n">
+        <v>166.38</v>
+      </c>
+      <c r="H838" t="n">
+        <v>158.91</v>
+      </c>
+      <c r="I838" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J838" t="b">
+        <v>0</v>
+      </c>
+      <c r="K838" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 166.50 &lt;= Upper 188.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>APP</t>
+        </is>
+      </c>
+      <c r="D839" t="n">
+        <v>323.96</v>
+      </c>
+      <c r="E839" t="n">
+        <v>323.6</v>
+      </c>
+      <c r="F839" t="n">
+        <v>323.6</v>
+      </c>
+      <c r="G839" t="n">
+        <v>315.29</v>
+      </c>
+      <c r="H839" t="n">
+        <v>323.99</v>
+      </c>
+      <c r="I839" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J839" t="b">
+        <v>0</v>
+      </c>
+      <c r="K839" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 315.29 &lt;= EMA21 323.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="D840" t="n">
+        <v>479.34</v>
+      </c>
+      <c r="E840" t="n">
+        <v>680.87</v>
+      </c>
+      <c r="F840" t="n">
+        <v>680.87</v>
+      </c>
+      <c r="G840" t="n">
+        <v>513.5</v>
+      </c>
+      <c r="H840" t="n">
+        <v>543.88</v>
+      </c>
+      <c r="I840" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J840" t="b">
+        <v>0</v>
+      </c>
+      <c r="K840" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 513.50 &lt;= EMA21 543.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="D841" t="n">
+        <v>289.37</v>
+      </c>
+      <c r="E841" t="n">
+        <v>353.1</v>
+      </c>
+      <c r="F841" t="n">
+        <v>353.1</v>
+      </c>
+      <c r="G841" t="n">
+        <v>298.04</v>
+      </c>
+      <c r="H841" t="n">
+        <v>311.6</v>
+      </c>
+      <c r="I841" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J841" t="b">
+        <v>0</v>
+      </c>
+      <c r="K841" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 298.04 &lt;= EMA21 311.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="D842" t="n">
+        <v>397.38</v>
+      </c>
+      <c r="E842" t="n">
+        <v>449.28</v>
+      </c>
+      <c r="F842" t="n">
+        <v>449.28</v>
+      </c>
+      <c r="G842" t="n">
+        <v>403.64</v>
+      </c>
+      <c r="H842" t="n">
+        <v>407.99</v>
+      </c>
+      <c r="I842" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J842" t="b">
+        <v>0</v>
+      </c>
+      <c r="K842" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 403.64 &lt;= EMA21 407.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>ADSK</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>212.4</v>
+      </c>
+      <c r="E843" t="n">
+        <v>279.64</v>
+      </c>
+      <c r="F843" t="n">
+        <v>279.64</v>
+      </c>
+      <c r="G843" t="n">
+        <v>224.07</v>
+      </c>
+      <c r="H843" t="n">
+        <v>234.01</v>
+      </c>
+      <c r="I843" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J843" t="b">
+        <v>0</v>
+      </c>
+      <c r="K843" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 224.07 &lt;= EMA21 234.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>ANSS</t>
+        </is>
+      </c>
+      <c r="J844" t="b">
+        <v>0</v>
+      </c>
+      <c r="K844" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+      <c r="D845" t="n">
+        <v>130.78</v>
+      </c>
+      <c r="E845" t="n">
+        <v>166.51</v>
+      </c>
+      <c r="F845" t="n">
+        <v>166.51</v>
+      </c>
+      <c r="G845" t="n">
+        <v>138.35</v>
+      </c>
+      <c r="H845" t="n">
+        <v>142.69</v>
+      </c>
+      <c r="I845" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J845" t="b">
+        <v>0</v>
+      </c>
+      <c r="K845" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 138.35 &lt;= EMA21 142.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>TYL</t>
+        </is>
+      </c>
+      <c r="D846" t="n">
+        <v>336.67</v>
+      </c>
+      <c r="E846" t="n">
+        <v>388.65</v>
+      </c>
+      <c r="F846" t="n">
+        <v>388.65</v>
+      </c>
+      <c r="G846" t="n">
+        <v>350.72</v>
+      </c>
+      <c r="H846" t="n">
+        <v>348.3</v>
+      </c>
+      <c r="I846" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J846" t="b">
+        <v>0</v>
+      </c>
+      <c r="K846" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 336.67 &lt;= Upper 388.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+      <c r="D847" t="n">
+        <v>141.66</v>
+      </c>
+      <c r="E847" t="n">
+        <v>161.97</v>
+      </c>
+      <c r="F847" t="n">
+        <v>161.97</v>
+      </c>
+      <c r="G847" t="n">
+        <v>147.27</v>
+      </c>
+      <c r="H847" t="n">
+        <v>147.98</v>
+      </c>
+      <c r="I847" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J847" t="b">
+        <v>0</v>
+      </c>
+      <c r="K847" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 147.27 &lt;= EMA21 147.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D848" t="n">
+        <v>179.59</v>
+      </c>
+      <c r="E848" t="n">
+        <v>207.89</v>
+      </c>
+      <c r="F848" t="n">
+        <v>207.89</v>
+      </c>
+      <c r="G848" t="n">
+        <v>181.1</v>
+      </c>
+      <c r="H848" t="n">
+        <v>182.47</v>
+      </c>
+      <c r="I848" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J848" t="b">
+        <v>0</v>
+      </c>
+      <c r="K848" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 181.10 &lt;= EMA21 182.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>CTSH</t>
+        </is>
+      </c>
+      <c r="D849" t="n">
+        <v>60</v>
+      </c>
+      <c r="E849" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="F849" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="G849" t="n">
+        <v>60.71</v>
+      </c>
+      <c r="H849" t="n">
+        <v>60.07</v>
+      </c>
+      <c r="I849" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J849" t="b">
+        <v>0</v>
+      </c>
+      <c r="K849" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 60.00 &lt;= Upper 66.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D850" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="E850" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="F850" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="G850" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="H850" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="I850" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J850" t="b">
+        <v>0</v>
+      </c>
+      <c r="K850" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11.39 &lt;= EMA21 11.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D851" t="n">
+        <v>117.91</v>
+      </c>
+      <c r="E851" t="n">
+        <v>124.21</v>
+      </c>
+      <c r="F851" t="n">
+        <v>124.21</v>
+      </c>
+      <c r="G851" t="n">
+        <v>115.54</v>
+      </c>
+      <c r="H851" t="n">
+        <v>111.74</v>
+      </c>
+      <c r="I851" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J851" t="b">
+        <v>0</v>
+      </c>
+      <c r="K851" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 117.91 &lt;= Upper 124.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>GEN</t>
+        </is>
+      </c>
+      <c r="D852" t="n">
+        <v>30.26</v>
+      </c>
+      <c r="E852" t="n">
+        <v>31.98</v>
+      </c>
+      <c r="F852" t="n">
+        <v>31.98</v>
+      </c>
+      <c r="G852" t="n">
+        <v>30.14</v>
+      </c>
+      <c r="H852" t="n">
+        <v>29.61</v>
+      </c>
+      <c r="I852" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J852" t="b">
+        <v>0</v>
+      </c>
+      <c r="K852" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 30.26 &lt;= Upper 31.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>CDW</t>
+        </is>
+      </c>
+      <c r="D853" t="n">
+        <v>153.79</v>
+      </c>
+      <c r="E853" t="n">
+        <v>157.92</v>
+      </c>
+      <c r="F853" t="n">
+        <v>157.92</v>
+      </c>
+      <c r="G853" t="n">
+        <v>147.34</v>
+      </c>
+      <c r="H853" t="n">
+        <v>144.7</v>
+      </c>
+      <c r="I853" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J853" t="b">
+        <v>0</v>
+      </c>
+      <c r="K853" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 153.79 &lt;= Upper 157.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>FFIV</t>
+        </is>
+      </c>
+      <c r="D854" t="n">
+        <v>411.71</v>
+      </c>
+      <c r="E854" t="n">
+        <v>414.09</v>
+      </c>
+      <c r="F854" t="n">
+        <v>414.09</v>
+      </c>
+      <c r="G854" t="n">
+        <v>399.23</v>
+      </c>
+      <c r="H854" t="n">
+        <v>398.18</v>
+      </c>
+      <c r="I854" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J854" t="b">
+        <v>0</v>
+      </c>
+      <c r="K854" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 411.71 &lt;= Upper 414.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>JNPR</t>
+        </is>
+      </c>
+      <c r="J855" t="b">
+        <v>0</v>
+      </c>
+      <c r="K855" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>AKAM</t>
+        </is>
+      </c>
+      <c r="D856" t="n">
+        <v>106.79</v>
+      </c>
+      <c r="E856" t="n">
+        <v>120.97</v>
+      </c>
+      <c r="F856" t="n">
+        <v>120.97</v>
+      </c>
+      <c r="G856" t="n">
+        <v>107.53</v>
+      </c>
+      <c r="H856" t="n">
+        <v>109.86</v>
+      </c>
+      <c r="I856" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J856" t="b">
+        <v>0</v>
+      </c>
+      <c r="K856" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 107.53 &lt;= EMA21 109.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="J857" t="b">
+        <v>0</v>
+      </c>
+      <c r="K857" t="inlineStr">
+        <is>
+          <t>INSUFFICIENT_DATA (&lt; 30 bars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>TTWO</t>
+        </is>
+      </c>
+      <c r="D858" t="n">
+        <v>215.47</v>
+      </c>
+      <c r="E858" t="n">
+        <v>251.84</v>
+      </c>
+      <c r="F858" t="n">
+        <v>251.84</v>
+      </c>
+      <c r="G858" t="n">
+        <v>217.81</v>
+      </c>
+      <c r="H858" t="n">
+        <v>225.14</v>
+      </c>
+      <c r="I858" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J858" t="b">
+        <v>0</v>
+      </c>
+      <c r="K858" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 217.81 &lt;= EMA21 225.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>RBLX</t>
+        </is>
+      </c>
+      <c r="D859" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="E859" t="n">
+        <v>45.96</v>
+      </c>
+      <c r="F859" t="n">
+        <v>45.96</v>
+      </c>
+      <c r="G859" t="n">
+        <v>43.24</v>
+      </c>
+      <c r="H859" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="I859" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J859" t="b">
+        <v>0</v>
+      </c>
+      <c r="K859" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 45.50 &lt;= Upper 45.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D860" t="n">
+        <v>43.96</v>
+      </c>
+      <c r="E860" t="n">
+        <v>48.27</v>
+      </c>
+      <c r="F860" t="n">
+        <v>48.27</v>
+      </c>
+      <c r="G860" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="H860" t="n">
+        <v>42.28</v>
+      </c>
+      <c r="I860" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J860" t="b">
+        <v>0</v>
+      </c>
+      <c r="K860" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 43.96 &lt;= Upper 48.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D861" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="E861" t="n">
+        <v>83.95</v>
+      </c>
+      <c r="F861" t="n">
+        <v>83.95</v>
+      </c>
+      <c r="G861" t="n">
+        <v>78.26000000000001</v>
+      </c>
+      <c r="H861" t="n">
+        <v>78.31999999999999</v>
+      </c>
+      <c r="I861" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J861" t="b">
+        <v>0</v>
+      </c>
+      <c r="K861" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 78.26 &lt;= EMA21 78.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D862" t="n">
+        <v>106.55</v>
+      </c>
+      <c r="E862" t="n">
+        <v>111.02</v>
+      </c>
+      <c r="F862" t="n">
+        <v>111.02</v>
+      </c>
+      <c r="G862" t="n">
+        <v>106.17</v>
+      </c>
+      <c r="H862" t="n">
+        <v>105.73</v>
+      </c>
+      <c r="I862" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J862" t="b">
+        <v>0</v>
+      </c>
+      <c r="K862" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 106.55 &lt;= Upper 111.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>WBD</t>
+        </is>
+      </c>
+      <c r="D863" t="n">
+        <v>28.04</v>
+      </c>
+      <c r="E863" t="n">
+        <v>29.01</v>
+      </c>
+      <c r="F863" t="n">
+        <v>29.01</v>
+      </c>
+      <c r="G863" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="H863" t="n">
+        <v>28.07</v>
+      </c>
+      <c r="I863" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J863" t="b">
+        <v>0</v>
+      </c>
+      <c r="K863" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 28.04 &lt;= Upper 29.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>PARA</t>
+        </is>
+      </c>
+      <c r="D864" t="n">
+        <v>1</v>
+      </c>
+      <c r="E864" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="F864" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="G864" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="H864" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I864" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J864" t="b">
+        <v>0</v>
+      </c>
+      <c r="K864" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1.06 &lt;= EMA21 1.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D865" t="n">
+        <v>525.75</v>
+      </c>
+      <c r="E865" t="n">
+        <v>567.67</v>
+      </c>
+      <c r="F865" t="n">
+        <v>567.67</v>
+      </c>
+      <c r="G865" t="n">
+        <v>532.9400000000001</v>
+      </c>
+      <c r="H865" t="n">
+        <v>528.98</v>
+      </c>
+      <c r="I865" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J865" t="b">
+        <v>0</v>
+      </c>
+      <c r="K865" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 525.75 &lt;= Upper 567.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>TME</t>
+        </is>
+      </c>
+      <c r="D866" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="E866" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="F866" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="G866" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="H866" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="I866" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="J866" t="b">
+        <v>0</v>
+      </c>
+      <c r="K866" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8.15 &lt;= EMA21 8.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="D867" t="n">
+        <v>107.15</v>
+      </c>
+      <c r="E867" t="n">
+        <v>115.22</v>
+      </c>
+      <c r="F867" t="n">
+        <v>115.22</v>
+      </c>
+      <c r="G867" t="n">
+        <v>106.39</v>
+      </c>
+      <c r="H867" t="n">
+        <v>107.43</v>
+      </c>
+      <c r="I867" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J867" t="b">
+        <v>0</v>
+      </c>
+      <c r="K867" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.39 &lt;= EMA21 107.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D868" t="n">
+        <v>904.77</v>
+      </c>
+      <c r="E868" t="n">
+        <v>981.22</v>
+      </c>
+      <c r="F868" t="n">
+        <v>981.22</v>
+      </c>
+      <c r="G868" t="n">
+        <v>917.0599999999999</v>
+      </c>
+      <c r="H868" t="n">
+        <v>930.58</v>
+      </c>
+      <c r="I868" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J868" t="b">
+        <v>0</v>
+      </c>
+      <c r="K868" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 917.06 &lt;= EMA21 930.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="D869" t="n">
+        <v>155.83</v>
+      </c>
+      <c r="E869" t="n">
+        <v>170.74</v>
+      </c>
+      <c r="F869" t="n">
+        <v>170.74</v>
+      </c>
+      <c r="G869" t="n">
+        <v>159.7</v>
+      </c>
+      <c r="H869" t="n">
+        <v>158.44</v>
+      </c>
+      <c r="I869" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J869" t="b">
+        <v>0</v>
+      </c>
+      <c r="K869" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 155.83 &lt;= Upper 170.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="D870" t="n">
+        <v>308.74</v>
+      </c>
+      <c r="E870" t="n">
+        <v>346.79</v>
+      </c>
+      <c r="F870" t="n">
+        <v>346.79</v>
+      </c>
+      <c r="G870" t="n">
+        <v>315.12</v>
+      </c>
+      <c r="H870" t="n">
+        <v>323.12</v>
+      </c>
+      <c r="I870" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J870" t="b">
+        <v>0</v>
+      </c>
+      <c r="K870" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 315.12 &lt;= EMA21 323.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D871" t="n">
+        <v>196.82</v>
+      </c>
+      <c r="E871" t="n">
+        <v>224.36</v>
+      </c>
+      <c r="F871" t="n">
+        <v>224.36</v>
+      </c>
+      <c r="G871" t="n">
+        <v>201.05</v>
+      </c>
+      <c r="H871" t="n">
+        <v>205.96</v>
+      </c>
+      <c r="I871" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J871" t="b">
+        <v>0</v>
+      </c>
+      <c r="K871" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 201.05 &lt;= EMA21 205.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D872" t="n">
+        <v>58.49</v>
+      </c>
+      <c r="E872" t="n">
+        <v>59.42</v>
+      </c>
+      <c r="F872" t="n">
+        <v>59.42</v>
+      </c>
+      <c r="G872" t="n">
+        <v>57.66</v>
+      </c>
+      <c r="H872" t="n">
+        <v>57.57</v>
+      </c>
+      <c r="I872" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="J872" t="b">
+        <v>0</v>
+      </c>
+      <c r="K872" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 58.49 &lt;= Upper 59.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="D873" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="E873" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="F873" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="G873" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="H873" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="I873" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J873" t="b">
+        <v>0</v>
+      </c>
+      <c r="K873" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12.15 &lt;= EMA21 12.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+      <c r="D874" t="n">
+        <v>124.58</v>
+      </c>
+      <c r="E874" t="n">
+        <v>132.88</v>
+      </c>
+      <c r="F874" t="n">
+        <v>132.88</v>
+      </c>
+      <c r="G874" t="n">
+        <v>126.31</v>
+      </c>
+      <c r="H874" t="n">
+        <v>125.62</v>
+      </c>
+      <c r="I874" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J874" t="b">
+        <v>0</v>
+      </c>
+      <c r="K874" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 124.58 &lt;= Upper 132.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>DLTR</t>
+        </is>
+      </c>
+      <c r="D875" t="n">
+        <v>118.17</v>
+      </c>
+      <c r="E875" t="n">
+        <v>138.97</v>
+      </c>
+      <c r="F875" t="n">
+        <v>138.97</v>
+      </c>
+      <c r="G875" t="n">
+        <v>124.02</v>
+      </c>
+      <c r="H875" t="n">
+        <v>126.68</v>
+      </c>
+      <c r="I875" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J875" t="b">
+        <v>0</v>
+      </c>
+      <c r="K875" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 124.02 &lt;= EMA21 126.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>BJ</t>
+        </is>
+      </c>
+      <c r="D876" t="n">
+        <v>91.48999999999999</v>
+      </c>
+      <c r="E876" t="n">
+        <v>97.15000000000001</v>
+      </c>
+      <c r="F876" t="n">
+        <v>97.15000000000001</v>
+      </c>
+      <c r="G876" t="n">
+        <v>91.14</v>
+      </c>
+      <c r="H876" t="n">
+        <v>92.14</v>
+      </c>
+      <c r="I876" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J876" t="b">
+        <v>0</v>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 91.14 &lt;= EMA21 92.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+      <c r="D877" t="n">
+        <v>230.74</v>
+      </c>
+      <c r="E877" t="n">
+        <v>243.5</v>
+      </c>
+      <c r="F877" t="n">
+        <v>243.5</v>
+      </c>
+      <c r="G877" t="n">
+        <v>229.46</v>
+      </c>
+      <c r="H877" t="n">
+        <v>232.79</v>
+      </c>
+      <c r="I877" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J877" t="b">
+        <v>0</v>
+      </c>
+      <c r="K877" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 229.46 &lt;= EMA21 232.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+      <c r="D878" t="n">
+        <v>126.02</v>
+      </c>
+      <c r="E878" t="n">
+        <v>152.99</v>
+      </c>
+      <c r="F878" t="n">
+        <v>152.99</v>
+      </c>
+      <c r="G878" t="n">
+        <v>130.05</v>
+      </c>
+      <c r="H878" t="n">
+        <v>136.47</v>
+      </c>
+      <c r="I878" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J878" t="b">
+        <v>0</v>
+      </c>
+      <c r="K878" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 130.05 &lt;= EMA21 136.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D879" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="E879" t="n">
+        <v>41.07</v>
+      </c>
+      <c r="F879" t="n">
+        <v>41.07</v>
+      </c>
+      <c r="G879" t="n">
+        <v>37.77</v>
+      </c>
+      <c r="H879" t="n">
+        <v>38.76</v>
+      </c>
+      <c r="I879" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J879" t="b">
+        <v>0</v>
+      </c>
+      <c r="K879" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 37.77 &lt;= EMA21 38.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D880" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="E880" t="n">
+        <v>131.7</v>
+      </c>
+      <c r="F880" t="n">
+        <v>131.7</v>
+      </c>
+      <c r="G880" t="n">
+        <v>106.08</v>
+      </c>
+      <c r="H880" t="n">
+        <v>112.08</v>
+      </c>
+      <c r="I880" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J880" t="b">
+        <v>0</v>
+      </c>
+      <c r="K880" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 106.08 &lt;= EMA21 112.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="D881" t="n">
+        <v>98.73999999999999</v>
+      </c>
+      <c r="E881" t="n">
+        <v>111.12</v>
+      </c>
+      <c r="F881" t="n">
+        <v>111.12</v>
+      </c>
+      <c r="G881" t="n">
+        <v>102.34</v>
+      </c>
+      <c r="H881" t="n">
+        <v>104.08</v>
+      </c>
+      <c r="I881" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J881" t="b">
+        <v>0</v>
+      </c>
+      <c r="K881" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 102.34 &lt;= EMA21 104.08)</t>
         </is>
       </c>
     </row>
@@ -33664,7 +37892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34133,6 +38361,130 @@
         <v>2.21</v>
       </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>88.34999999999999</v>
+      </c>
+      <c r="E16" t="n">
+        <v>84.37</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>QRVO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>116.65</v>
+      </c>
+      <c r="E17" t="n">
+        <v>111.4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>567.29</v>
+      </c>
+      <c r="E18" t="n">
+        <v>541.76</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="E19" t="n">
+        <v>33.88</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -34149,7 +38501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34230,19 +38582,19 @@
         <v>1961.07</v>
       </c>
       <c r="F2" t="n">
-        <v>653.6900000000001</v>
+        <v>648.03</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>-0.87</v>
       </c>
       <c r="H2" t="n">
-        <v>624.27</v>
+        <v>634.35</v>
       </c>
       <c r="I2" t="n">
-        <v>653.6900000000001</v>
+        <v>664.239990234375</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -34368,6 +38720,47 @@
         <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="D6" t="n">
+        <v>56</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1986.88</v>
+      </c>
+      <c r="F6" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>33.88</v>
+      </c>
+      <c r="I6" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -34771,7 +39164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35561,6 +39954,55 @@
         </is>
       </c>
       <c r="K16" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-12 04:45:33</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>35583981F4</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>HPQ</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="G17" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>56</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
         </is>
@@ -35577,7 +40019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35685,6 +40127,33 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>Opened at 104.36 below SL of 109.14. Filled at Open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-12 04:45:33</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SKIPPED_CAPITAL_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Qualified breakout on DELL skipped: all slots full or insufficient cash.</t>
         </is>
       </c>
     </row>
@@ -35699,7 +40168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36145,6 +40614,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>04:45:34</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>25.44</v>
+      </c>
+      <c r="D14" t="n">
+        <v>9736.440000000001</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9761.879999999999</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-238.12</v>
+      </c>
+      <c r="G14" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>